<commit_message>
Actualización mayo y tabla de resolutividad
</commit_message>
<xml_diff>
--- a/Dashboard.xlsx
+++ b/Dashboard.xlsx
@@ -5,10 +5,10 @@
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauricio\Desktop\NUEVO\Productividad2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauricio\Desktop\NUEVO\DashboardMedico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9AA829A-30F6-47F8-BC2C-C693875C58DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{729B26A0-31D1-4E96-98B4-8F27F0BD3923}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{1407A859-4935-4127-A91B-F2429559B5A8}"/>
   </bookViews>
@@ -23,7 +23,7 @@
   </definedNames>
   <calcPr calcId="181029"/>
   <pivotCaches>
-    <pivotCache cacheId="11" r:id="rId4"/>
+    <pivotCache cacheId="3" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="48">
   <si>
     <t>mes</t>
   </si>
@@ -184,6 +184,9 @@
   </si>
   <si>
     <t>Suma de % laboratorios</t>
+  </si>
+  <si>
+    <t>mayo</t>
   </si>
 </sst>
 </file>
@@ -909,10 +912,52 @@
     <xf numFmtId="10" fontId="4" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -925,48 +970,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -10274,359 +10277,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9343E3D3-8E4C-4B20-B961-BB4621992C8B}" name="TablaDinámica7" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
-  <location ref="I18:J23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="22">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item h="1" x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="11">
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item x="0"/>
-        <item h="1" x="6"/>
-        <item h="1" x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="8"/>
-        <item h="1" x="7"/>
-        <item h="1" x="3"/>
-        <item h="1" x="9"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Suma de % Rendimiento" fld="12" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="5" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{931E7B7E-CA9F-465C-B9CA-2A2FFF91B95F}" name="TablaDinámica6" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
-  <location ref="F18:G23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="22">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item h="1" x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="11">
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item x="0"/>
-        <item h="1" x="6"/>
-        <item h="1" x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="8"/>
-        <item h="1" x="7"/>
-        <item h="1" x="3"/>
-        <item h="1" x="9"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Suma de % Cumplimiento" fld="6" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="6" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E63473CF-27CE-4690-9F1E-A43D9330F8B0}" name="TablaDinámica5" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
-  <location ref="F11:I16" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="22">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item h="1" x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="11">
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item x="0"/>
-        <item h="1" x="6"/>
-        <item h="1" x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="8"/>
-        <item h="1" x="7"/>
-        <item h="1" x="3"/>
-        <item h="1" x="9"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
-  </colItems>
-  <dataFields count="3">
-    <dataField name="Suma de % formulas" fld="14" baseField="0" baseItem="0"/>
-    <dataField name="Suma de % laboratorios" fld="16" baseField="0" baseItem="0"/>
-    <dataField name="Suma de %Ayudas Diagnosticas" fld="18" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="5">
-    <chartFormat chart="6" format="21" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="22" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="23">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="24">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="25" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{84E442F7-39EA-4DAC-85E9-0D554B59BD1E}" name="TablaDinámica4" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{84E442F7-39EA-4DAC-85E9-0D554B59BD1E}" name="TablaDinámica4" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E3:L8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="22">
     <pivotField axis="axisRow" showAll="0">
@@ -10772,8 +10423,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8798F489-BE3A-43ED-960C-7BA2B41DFF28}" name="TablaDinámica8" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8798F489-BE3A-43ED-960C-7BA2B41DFF28}" name="TablaDinámica8" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
   <location ref="G26:I31" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="22">
     <pivotField axis="axisRow" showAll="0">
@@ -10902,6 +10553,358 @@
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
             <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9343E3D3-8E4C-4B20-B961-BB4621992C8B}" name="TablaDinámica7" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+  <location ref="I18:J23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="22">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item h="1" x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="11">
+        <item h="1" x="5"/>
+        <item h="1" x="4"/>
+        <item x="0"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="8"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="9"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Suma de % Rendimiento" fld="12" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{931E7B7E-CA9F-465C-B9CA-2A2FFF91B95F}" name="TablaDinámica6" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+  <location ref="F18:G23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="22">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item h="1" x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="11">
+        <item h="1" x="5"/>
+        <item h="1" x="4"/>
+        <item x="0"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="8"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="9"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Suma de % Cumplimiento" fld="6" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="6" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E63473CF-27CE-4690-9F1E-A43D9330F8B0}" name="TablaDinámica5" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+  <location ref="F11:I16" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="22">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item h="1" x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="11">
+        <item h="1" x="5"/>
+        <item h="1" x="4"/>
+        <item x="0"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="8"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="9"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+  </colItems>
+  <dataFields count="3">
+    <dataField name="Suma de % formulas" fld="14" baseField="0" baseItem="0"/>
+    <dataField name="Suma de % laboratorios" fld="16" baseField="0" baseItem="0"/>
+    <dataField name="Suma de %Ayudas Diagnosticas" fld="18" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="5">
+    <chartFormat chart="6" format="21" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="22" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="23">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="24">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="25" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="2"/>
           </reference>
         </references>
       </pivotArea>
@@ -11281,7 +11284,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4FD4F9-2910-4648-84AF-C941CDDEB3D5}">
-  <dimension ref="A1:V34"/>
+  <dimension ref="A1:V43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="11.42578125" style="60"/>
@@ -11322,10 +11325,10 @@
       <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="85" t="s">
+      <c r="K1" s="71" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="86"/>
+      <c r="L1" s="72"/>
       <c r="M1" s="63" t="s">
         <v>11</v>
       </c>
@@ -11392,10 +11395,10 @@
       <c r="J2" s="11">
         <v>70</v>
       </c>
-      <c r="K2" s="69">
+      <c r="K2" s="73">
         <v>11</v>
       </c>
-      <c r="L2" s="70"/>
+      <c r="L2" s="74"/>
       <c r="M2" s="64">
         <f>J2/I2</f>
         <v>0.86419753086419748</v>
@@ -11454,7 +11457,7 @@
         <v>2</v>
       </c>
       <c r="G3" s="64">
-        <f t="shared" ref="G3:G34" si="1">E3/D3</f>
+        <f t="shared" ref="G3:G43" si="1">E3/D3</f>
         <v>0.8</v>
       </c>
       <c r="H3" s="14">
@@ -11468,44 +11471,44 @@
       <c r="J3" s="16">
         <v>60</v>
       </c>
-      <c r="K3" s="79">
+      <c r="K3" s="75">
         <v>8</v>
       </c>
-      <c r="L3" s="80"/>
+      <c r="L3" s="76"/>
       <c r="M3" s="64">
-        <f t="shared" ref="M3:M34" si="3">J3/I3</f>
+        <f t="shared" ref="M3:M43" si="3">J3/I3</f>
         <v>0.88235294117647056</v>
       </c>
       <c r="N3" s="17">
         <v>55</v>
       </c>
       <c r="O3" s="66">
-        <f t="shared" ref="O3:O34" si="4">N3/J3</f>
+        <f t="shared" ref="O3:O43" si="4">N3/J3</f>
         <v>0.91666666666666663</v>
       </c>
       <c r="P3" s="16">
         <v>4</v>
       </c>
       <c r="Q3" s="66">
-        <f t="shared" ref="Q3:Q34" si="5">P3/J3</f>
+        <f t="shared" ref="Q3:Q43" si="5">P3/J3</f>
         <v>6.6666666666666666E-2</v>
       </c>
       <c r="R3" s="16">
         <v>2</v>
       </c>
       <c r="S3" s="67">
-        <f t="shared" ref="S3:S34" si="6">R3/J3</f>
+        <f t="shared" ref="S3:S43" si="6">R3/J3</f>
         <v>3.3333333333333333E-2</v>
       </c>
       <c r="T3" s="14">
         <v>7</v>
       </c>
       <c r="U3" s="66">
-        <f t="shared" ref="U3:U34" si="7">T3/J3</f>
+        <f t="shared" ref="U3:U43" si="7">T3/J3</f>
         <v>0.11666666666666667</v>
       </c>
       <c r="V3" s="68">
-        <f t="shared" ref="V3:V34" si="8">(1-(T3/J3))</f>
+        <f t="shared" ref="V3:V43" si="8">(1-(T3/J3))</f>
         <v>0.8833333333333333</v>
       </c>
     </row>
@@ -11544,10 +11547,10 @@
       <c r="J4" s="11">
         <v>50</v>
       </c>
-      <c r="K4" s="83">
+      <c r="K4" s="69">
         <v>10</v>
       </c>
-      <c r="L4" s="84"/>
+      <c r="L4" s="70"/>
       <c r="M4" s="64">
         <f t="shared" si="3"/>
         <v>0.83333333333333337</v>
@@ -11620,10 +11623,10 @@
       <c r="J5" s="11">
         <v>18</v>
       </c>
-      <c r="K5" s="83">
+      <c r="K5" s="69">
         <v>3</v>
       </c>
-      <c r="L5" s="84"/>
+      <c r="L5" s="70"/>
       <c r="M5" s="64">
         <f t="shared" si="3"/>
         <v>0.8571428571428571</v>
@@ -11772,10 +11775,10 @@
       <c r="J7" s="16">
         <v>10</v>
       </c>
-      <c r="K7" s="79">
+      <c r="K7" s="75">
         <v>1</v>
       </c>
-      <c r="L7" s="80"/>
+      <c r="L7" s="76"/>
       <c r="M7" s="64">
         <f t="shared" si="3"/>
         <v>0.90909090909090906</v>
@@ -11848,10 +11851,10 @@
       <c r="J8" s="27">
         <v>8</v>
       </c>
-      <c r="K8" s="87">
+      <c r="K8" s="79">
         <v>1</v>
       </c>
-      <c r="L8" s="88"/>
+      <c r="L8" s="80"/>
       <c r="M8" s="64">
         <f t="shared" si="3"/>
         <v>0.88888888888888884</v>
@@ -11924,10 +11927,10 @@
       <c r="J9" s="11">
         <v>139</v>
       </c>
-      <c r="K9" s="69">
+      <c r="K9" s="73">
         <v>4</v>
       </c>
-      <c r="L9" s="70"/>
+      <c r="L9" s="74"/>
       <c r="M9" s="64">
         <f t="shared" si="3"/>
         <v>0.97202797202797198</v>
@@ -12000,10 +12003,10 @@
       <c r="J10" s="16">
         <v>112</v>
       </c>
-      <c r="K10" s="79">
+      <c r="K10" s="75">
         <v>2</v>
       </c>
-      <c r="L10" s="80"/>
+      <c r="L10" s="76"/>
       <c r="M10" s="64">
         <f t="shared" si="3"/>
         <v>0.98245614035087714</v>
@@ -12076,10 +12079,10 @@
       <c r="J11" s="11">
         <v>77</v>
       </c>
-      <c r="K11" s="83">
+      <c r="K11" s="69">
         <v>1</v>
       </c>
-      <c r="L11" s="84"/>
+      <c r="L11" s="70"/>
       <c r="M11" s="64">
         <f t="shared" si="3"/>
         <v>0.98717948717948723</v>
@@ -12152,10 +12155,10 @@
       <c r="J12" s="11">
         <v>61</v>
       </c>
-      <c r="K12" s="83">
+      <c r="K12" s="69">
         <v>4</v>
       </c>
-      <c r="L12" s="84"/>
+      <c r="L12" s="70"/>
       <c r="M12" s="64">
         <f t="shared" si="3"/>
         <v>0.93846153846153846</v>
@@ -12304,10 +12307,10 @@
       <c r="J14" s="16">
         <v>21</v>
       </c>
-      <c r="K14" s="79">
+      <c r="K14" s="75">
         <v>1</v>
       </c>
-      <c r="L14" s="80"/>
+      <c r="L14" s="76"/>
       <c r="M14" s="64">
         <f t="shared" si="3"/>
         <v>0.95454545454545459</v>
@@ -12379,10 +12382,10 @@
       <c r="J15" s="34">
         <v>28</v>
       </c>
-      <c r="K15" s="75">
+      <c r="K15" s="81">
         <v>0</v>
       </c>
-      <c r="L15" s="76"/>
+      <c r="L15" s="82"/>
       <c r="M15" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -12455,10 +12458,10 @@
       <c r="J16" s="40">
         <v>23</v>
       </c>
-      <c r="K16" s="81">
+      <c r="K16" s="83">
         <v>1</v>
       </c>
-      <c r="L16" s="82"/>
+      <c r="L16" s="84"/>
       <c r="M16" s="64">
         <f t="shared" si="3"/>
         <v>0.95833333333333337</v>
@@ -12531,10 +12534,10 @@
       <c r="J17" s="11">
         <v>164</v>
       </c>
-      <c r="K17" s="69">
+      <c r="K17" s="73">
         <v>2</v>
       </c>
-      <c r="L17" s="70"/>
+      <c r="L17" s="74"/>
       <c r="M17" s="64">
         <f t="shared" si="3"/>
         <v>0.98795180722891562</v>
@@ -12607,10 +12610,10 @@
       <c r="J18" s="16">
         <v>133</v>
       </c>
-      <c r="K18" s="79">
+      <c r="K18" s="75">
         <v>2</v>
       </c>
-      <c r="L18" s="80"/>
+      <c r="L18" s="76"/>
       <c r="M18" s="64">
         <f t="shared" si="3"/>
         <v>0.98518518518518516</v>
@@ -12683,10 +12686,10 @@
       <c r="J19" s="11">
         <v>111</v>
       </c>
-      <c r="K19" s="83">
+      <c r="K19" s="69">
         <v>1</v>
       </c>
-      <c r="L19" s="84"/>
+      <c r="L19" s="70"/>
       <c r="M19" s="64">
         <f t="shared" si="3"/>
         <v>0.9910714285714286</v>
@@ -12759,10 +12762,10 @@
       <c r="J20" s="11">
         <v>76</v>
       </c>
-      <c r="K20" s="83">
+      <c r="K20" s="69">
         <v>1</v>
       </c>
-      <c r="L20" s="84"/>
+      <c r="L20" s="70"/>
       <c r="M20" s="64">
         <f t="shared" si="3"/>
         <v>0.98701298701298701</v>
@@ -12834,10 +12837,10 @@
       <c r="J21" s="11">
         <v>43</v>
       </c>
-      <c r="K21" s="83">
+      <c r="K21" s="69">
         <v>2</v>
       </c>
-      <c r="L21" s="84"/>
+      <c r="L21" s="70"/>
       <c r="M21" s="64">
         <f t="shared" si="3"/>
         <v>0.9555555555555556</v>
@@ -12986,10 +12989,10 @@
       <c r="J23" s="16">
         <v>26</v>
       </c>
-      <c r="K23" s="79">
+      <c r="K23" s="75">
         <v>1</v>
       </c>
-      <c r="L23" s="80"/>
+      <c r="L23" s="76"/>
       <c r="M23" s="64">
         <f t="shared" si="3"/>
         <v>0.96296296296296291</v>
@@ -13061,10 +13064,10 @@
       <c r="J24" s="34">
         <v>30</v>
       </c>
-      <c r="K24" s="75">
+      <c r="K24" s="81">
         <v>0</v>
       </c>
-      <c r="L24" s="76"/>
+      <c r="L24" s="82"/>
       <c r="M24" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -13137,10 +13140,10 @@
       <c r="J25" s="49">
         <v>43</v>
       </c>
-      <c r="K25" s="71">
+      <c r="K25" s="85">
         <v>2</v>
       </c>
-      <c r="L25" s="72"/>
+      <c r="L25" s="86"/>
       <c r="M25" s="64">
         <f t="shared" si="3"/>
         <v>0.9555555555555556</v>
@@ -13212,11 +13215,11 @@
       <c r="J26" s="56">
         <v>143</v>
       </c>
-      <c r="K26" s="73">
+      <c r="K26" s="87">
         <f>I26-J26</f>
         <v>6</v>
       </c>
-      <c r="L26" s="74"/>
+      <c r="L26" s="88"/>
       <c r="M26" s="64">
         <f t="shared" si="3"/>
         <v>0.95973154362416102</v>
@@ -13288,11 +13291,11 @@
       <c r="J27" s="16">
         <v>74</v>
       </c>
-      <c r="K27" s="69">
+      <c r="K27" s="73">
         <f>I27-J27</f>
         <v>1</v>
       </c>
-      <c r="L27" s="70"/>
+      <c r="L27" s="74"/>
       <c r="M27" s="64">
         <f t="shared" si="3"/>
         <v>0.98666666666666669</v>
@@ -13364,11 +13367,11 @@
       <c r="J28" s="11">
         <v>83</v>
       </c>
-      <c r="K28" s="69">
+      <c r="K28" s="73">
         <f t="shared" ref="K28:K29" si="20">I28-J28</f>
         <v>0</v>
       </c>
-      <c r="L28" s="70"/>
+      <c r="L28" s="74"/>
       <c r="M28" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -13440,11 +13443,11 @@
       <c r="J29" s="11">
         <v>79</v>
       </c>
-      <c r="K29" s="69">
+      <c r="K29" s="73">
         <f t="shared" si="20"/>
         <v>3</v>
       </c>
-      <c r="L29" s="70"/>
+      <c r="L29" s="74"/>
       <c r="M29" s="64">
         <f t="shared" si="3"/>
         <v>0.96341463414634143</v>
@@ -13516,11 +13519,11 @@
       <c r="J30" s="11">
         <v>93</v>
       </c>
-      <c r="K30" s="69">
+      <c r="K30" s="73">
         <f>I30-J30</f>
         <v>0</v>
       </c>
-      <c r="L30" s="70"/>
+      <c r="L30" s="74"/>
       <c r="M30" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -13592,11 +13595,11 @@
       <c r="J31" s="20">
         <v>78</v>
       </c>
-      <c r="K31" s="69">
+      <c r="K31" s="73">
         <f>I31-J31</f>
         <v>1</v>
       </c>
-      <c r="L31" s="70"/>
+      <c r="L31" s="74"/>
       <c r="M31" s="64">
         <f t="shared" si="3"/>
         <v>0.98734177215189878</v>
@@ -13668,11 +13671,11 @@
       <c r="J32" s="16">
         <v>33</v>
       </c>
-      <c r="K32" s="69">
+      <c r="K32" s="73">
         <f t="shared" ref="K32:K33" si="22">I32-J32</f>
         <v>0</v>
       </c>
-      <c r="L32" s="70"/>
+      <c r="L32" s="74"/>
       <c r="M32" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -13744,11 +13747,11 @@
       <c r="J33" s="34">
         <v>28</v>
       </c>
-      <c r="K33" s="69">
+      <c r="K33" s="73">
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
-      <c r="L33" s="70"/>
+      <c r="L33" s="74"/>
       <c r="M33" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -13820,11 +13823,11 @@
       <c r="J34" s="49">
         <v>35</v>
       </c>
-      <c r="K34" s="69">
+      <c r="K34" s="73">
         <f>I34-J34</f>
         <v>2</v>
       </c>
-      <c r="L34" s="70"/>
+      <c r="L34" s="74"/>
       <c r="M34" s="64">
         <f t="shared" si="3"/>
         <v>0.94594594594594594</v>
@@ -13862,8 +13865,678 @@
         <v>1</v>
       </c>
     </row>
+    <row r="35" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>47</v>
+      </c>
+      <c r="B35" t="s">
+        <v>22</v>
+      </c>
+      <c r="C35" t="s">
+        <v>23</v>
+      </c>
+      <c r="D35">
+        <v>18</v>
+      </c>
+      <c r="E35">
+        <v>17</v>
+      </c>
+      <c r="F35">
+        <v>1</v>
+      </c>
+      <c r="G35" s="64">
+        <f t="shared" si="1"/>
+        <v>0.94444444444444442</v>
+      </c>
+      <c r="H35">
+        <v>204</v>
+      </c>
+      <c r="I35">
+        <v>161</v>
+      </c>
+      <c r="J35">
+        <v>134</v>
+      </c>
+      <c r="K35">
+        <v>27</v>
+      </c>
+      <c r="M35" s="64">
+        <f t="shared" si="3"/>
+        <v>0.83229813664596275</v>
+      </c>
+      <c r="N35">
+        <v>83</v>
+      </c>
+      <c r="O35" s="66">
+        <f t="shared" si="4"/>
+        <v>0.61940298507462688</v>
+      </c>
+      <c r="P35">
+        <v>21</v>
+      </c>
+      <c r="Q35" s="66">
+        <f t="shared" si="5"/>
+        <v>0.15671641791044777</v>
+      </c>
+      <c r="R35">
+        <v>10</v>
+      </c>
+      <c r="S35" s="67">
+        <f t="shared" si="6"/>
+        <v>7.4626865671641784E-2</v>
+      </c>
+      <c r="T35">
+        <v>21</v>
+      </c>
+      <c r="U35" s="66">
+        <f t="shared" si="7"/>
+        <v>0.15671641791044777</v>
+      </c>
+      <c r="V35" s="68">
+        <f t="shared" si="8"/>
+        <v>0.84328358208955223</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>47</v>
+      </c>
+      <c r="B36" t="s">
+        <v>22</v>
+      </c>
+      <c r="C36" t="s">
+        <v>24</v>
+      </c>
+      <c r="D36">
+        <v>19</v>
+      </c>
+      <c r="E36">
+        <v>19</v>
+      </c>
+      <c r="F36">
+        <v>0</v>
+      </c>
+      <c r="G36" s="64">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H36">
+        <v>152</v>
+      </c>
+      <c r="I36">
+        <v>151</v>
+      </c>
+      <c r="J36">
+        <v>118</v>
+      </c>
+      <c r="K36">
+        <v>33</v>
+      </c>
+      <c r="M36" s="64">
+        <f t="shared" si="3"/>
+        <v>0.7814569536423841</v>
+      </c>
+      <c r="N36">
+        <v>88</v>
+      </c>
+      <c r="O36" s="66">
+        <f t="shared" si="4"/>
+        <v>0.74576271186440679</v>
+      </c>
+      <c r="P36">
+        <v>19</v>
+      </c>
+      <c r="Q36" s="66">
+        <f t="shared" si="5"/>
+        <v>0.16101694915254236</v>
+      </c>
+      <c r="R36">
+        <v>20</v>
+      </c>
+      <c r="S36" s="67">
+        <f t="shared" si="6"/>
+        <v>0.16949152542372881</v>
+      </c>
+      <c r="T36">
+        <v>25</v>
+      </c>
+      <c r="U36" s="66">
+        <f t="shared" si="7"/>
+        <v>0.21186440677966101</v>
+      </c>
+      <c r="V36" s="68">
+        <f t="shared" si="8"/>
+        <v>0.78813559322033899</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>47</v>
+      </c>
+      <c r="B37" t="s">
+        <v>22</v>
+      </c>
+      <c r="C37" t="s">
+        <v>25</v>
+      </c>
+      <c r="D37">
+        <v>19</v>
+      </c>
+      <c r="E37">
+        <v>17</v>
+      </c>
+      <c r="F37">
+        <v>2</v>
+      </c>
+      <c r="G37" s="64">
+        <f t="shared" si="1"/>
+        <v>0.89473684210526316</v>
+      </c>
+      <c r="H37">
+        <v>136</v>
+      </c>
+      <c r="I37">
+        <v>126</v>
+      </c>
+      <c r="J37">
+        <v>86</v>
+      </c>
+      <c r="K37">
+        <v>40</v>
+      </c>
+      <c r="M37" s="64">
+        <f t="shared" si="3"/>
+        <v>0.68253968253968256</v>
+      </c>
+      <c r="N37">
+        <v>78</v>
+      </c>
+      <c r="O37" s="66">
+        <f t="shared" si="4"/>
+        <v>0.90697674418604646</v>
+      </c>
+      <c r="P37">
+        <v>3</v>
+      </c>
+      <c r="Q37" s="66">
+        <f t="shared" si="5"/>
+        <v>3.4883720930232558E-2</v>
+      </c>
+      <c r="R37">
+        <v>5</v>
+      </c>
+      <c r="S37" s="67">
+        <f t="shared" si="6"/>
+        <v>5.8139534883720929E-2</v>
+      </c>
+      <c r="T37">
+        <v>10</v>
+      </c>
+      <c r="U37" s="66">
+        <f t="shared" si="7"/>
+        <v>0.11627906976744186</v>
+      </c>
+      <c r="V37" s="68">
+        <f t="shared" si="8"/>
+        <v>0.88372093023255816</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>47</v>
+      </c>
+      <c r="B38" t="s">
+        <v>22</v>
+      </c>
+      <c r="C38" t="s">
+        <v>26</v>
+      </c>
+      <c r="D38">
+        <v>19</v>
+      </c>
+      <c r="E38">
+        <v>17</v>
+      </c>
+      <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38" s="64">
+        <f t="shared" si="1"/>
+        <v>0.89473684210526316</v>
+      </c>
+      <c r="H38">
+        <v>136</v>
+      </c>
+      <c r="I38">
+        <v>126</v>
+      </c>
+      <c r="J38">
+        <v>91</v>
+      </c>
+      <c r="K38">
+        <v>35</v>
+      </c>
+      <c r="M38" s="64">
+        <f t="shared" si="3"/>
+        <v>0.72222222222222221</v>
+      </c>
+      <c r="N38">
+        <v>81</v>
+      </c>
+      <c r="O38" s="66">
+        <f t="shared" si="4"/>
+        <v>0.89010989010989006</v>
+      </c>
+      <c r="P38">
+        <v>8</v>
+      </c>
+      <c r="Q38" s="66">
+        <f t="shared" si="5"/>
+        <v>8.7912087912087919E-2</v>
+      </c>
+      <c r="R38">
+        <v>3</v>
+      </c>
+      <c r="S38" s="67">
+        <f t="shared" si="6"/>
+        <v>3.2967032967032968E-2</v>
+      </c>
+      <c r="T38">
+        <v>11</v>
+      </c>
+      <c r="U38" s="66">
+        <f t="shared" si="7"/>
+        <v>0.12087912087912088</v>
+      </c>
+      <c r="V38" s="68">
+        <f t="shared" si="8"/>
+        <v>0.87912087912087911</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>47</v>
+      </c>
+      <c r="B39" t="s">
+        <v>35</v>
+      </c>
+      <c r="C39" t="s">
+        <v>36</v>
+      </c>
+      <c r="D39">
+        <v>16</v>
+      </c>
+      <c r="E39">
+        <v>15</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="G39" s="64">
+        <f t="shared" si="1"/>
+        <v>0.9375</v>
+      </c>
+      <c r="H39">
+        <v>90</v>
+      </c>
+      <c r="I39">
+        <v>130</v>
+      </c>
+      <c r="J39">
+        <v>92</v>
+      </c>
+      <c r="K39">
+        <v>38</v>
+      </c>
+      <c r="M39" s="64">
+        <f t="shared" si="3"/>
+        <v>0.70769230769230773</v>
+      </c>
+      <c r="N39">
+        <v>81</v>
+      </c>
+      <c r="O39" s="66">
+        <f t="shared" si="4"/>
+        <v>0.88043478260869568</v>
+      </c>
+      <c r="P39">
+        <v>101</v>
+      </c>
+      <c r="Q39" s="66">
+        <f t="shared" si="5"/>
+        <v>1.0978260869565217</v>
+      </c>
+      <c r="R39">
+        <v>47</v>
+      </c>
+      <c r="S39" s="67">
+        <f t="shared" si="6"/>
+        <v>0.51086956521739135</v>
+      </c>
+      <c r="T39">
+        <v>16</v>
+      </c>
+      <c r="U39" s="66">
+        <f t="shared" si="7"/>
+        <v>0.17391304347826086</v>
+      </c>
+      <c r="V39" s="68">
+        <f t="shared" si="8"/>
+        <v>0.82608695652173914</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>47</v>
+      </c>
+      <c r="B40" t="s">
+        <v>27</v>
+      </c>
+      <c r="C40" t="s">
+        <v>28</v>
+      </c>
+      <c r="D40">
+        <v>19</v>
+      </c>
+      <c r="E40">
+        <v>19</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40" s="64">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H40">
+        <v>304</v>
+      </c>
+      <c r="I40">
+        <v>76</v>
+      </c>
+      <c r="J40">
+        <v>53</v>
+      </c>
+      <c r="K40">
+        <v>23</v>
+      </c>
+      <c r="M40" s="64">
+        <f t="shared" si="3"/>
+        <v>0.69736842105263153</v>
+      </c>
+      <c r="N40">
+        <v>4</v>
+      </c>
+      <c r="O40" s="66">
+        <f t="shared" si="4"/>
+        <v>7.5471698113207544E-2</v>
+      </c>
+      <c r="P40">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="66">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R40">
+        <v>10</v>
+      </c>
+      <c r="S40" s="67">
+        <f t="shared" si="6"/>
+        <v>0.18867924528301888</v>
+      </c>
+      <c r="T40">
+        <v>4</v>
+      </c>
+      <c r="U40" s="66">
+        <f t="shared" si="7"/>
+        <v>7.5471698113207544E-2</v>
+      </c>
+      <c r="V40" s="68">
+        <f t="shared" si="8"/>
+        <v>0.92452830188679247</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>47</v>
+      </c>
+      <c r="B41" t="s">
+        <v>27</v>
+      </c>
+      <c r="C41" t="s">
+        <v>29</v>
+      </c>
+      <c r="D41">
+        <v>19</v>
+      </c>
+      <c r="E41">
+        <v>15</v>
+      </c>
+      <c r="F41">
+        <v>4</v>
+      </c>
+      <c r="G41" s="64">
+        <f t="shared" si="1"/>
+        <v>0.78947368421052633</v>
+      </c>
+      <c r="H41">
+        <v>120</v>
+      </c>
+      <c r="I41">
+        <v>34</v>
+      </c>
+      <c r="J41">
+        <v>29</v>
+      </c>
+      <c r="K41">
+        <v>5</v>
+      </c>
+      <c r="M41" s="64">
+        <f t="shared" si="3"/>
+        <v>0.8529411764705882</v>
+      </c>
+      <c r="N41">
+        <v>1</v>
+      </c>
+      <c r="O41" s="66">
+        <f t="shared" si="4"/>
+        <v>3.4482758620689655E-2</v>
+      </c>
+      <c r="P41">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="66">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R41">
+        <v>6</v>
+      </c>
+      <c r="S41" s="67">
+        <f t="shared" si="6"/>
+        <v>0.20689655172413793</v>
+      </c>
+      <c r="T41">
+        <v>0</v>
+      </c>
+      <c r="U41" s="66">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="V41" s="68">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>47</v>
+      </c>
+      <c r="B42" t="s">
+        <v>27</v>
+      </c>
+      <c r="C42" t="s">
+        <v>33</v>
+      </c>
+      <c r="D42">
+        <v>19</v>
+      </c>
+      <c r="E42">
+        <v>12</v>
+      </c>
+      <c r="F42">
+        <v>7</v>
+      </c>
+      <c r="G42" s="64">
+        <f t="shared" si="1"/>
+        <v>0.63157894736842102</v>
+      </c>
+      <c r="H42">
+        <v>96</v>
+      </c>
+      <c r="I42">
+        <v>29</v>
+      </c>
+      <c r="J42">
+        <v>22</v>
+      </c>
+      <c r="K42">
+        <v>7</v>
+      </c>
+      <c r="M42" s="64">
+        <f t="shared" si="3"/>
+        <v>0.75862068965517238</v>
+      </c>
+      <c r="N42">
+        <v>1</v>
+      </c>
+      <c r="O42" s="66">
+        <f t="shared" si="4"/>
+        <v>4.5454545454545456E-2</v>
+      </c>
+      <c r="P42">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="66">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R42">
+        <v>2</v>
+      </c>
+      <c r="S42" s="67">
+        <f t="shared" si="6"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+      <c r="T42">
+        <v>1</v>
+      </c>
+      <c r="U42" s="66">
+        <f t="shared" si="7"/>
+        <v>4.5454545454545456E-2</v>
+      </c>
+      <c r="V42" s="68">
+        <f t="shared" si="8"/>
+        <v>0.95454545454545459</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>47</v>
+      </c>
+      <c r="B43" t="s">
+        <v>30</v>
+      </c>
+      <c r="C43" t="s">
+        <v>31</v>
+      </c>
+      <c r="D43">
+        <v>14</v>
+      </c>
+      <c r="E43">
+        <v>14</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43" s="64">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H43">
+        <v>112</v>
+      </c>
+      <c r="I43">
+        <v>60</v>
+      </c>
+      <c r="J43">
+        <v>40</v>
+      </c>
+      <c r="K43">
+        <v>20</v>
+      </c>
+      <c r="M43" s="64">
+        <f t="shared" si="3"/>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="N43">
+        <v>0</v>
+      </c>
+      <c r="O43" s="66">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="P43">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="66">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R43">
+        <v>0</v>
+      </c>
+      <c r="S43" s="67">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="T43">
+        <v>1</v>
+      </c>
+      <c r="U43" s="66">
+        <f t="shared" si="7"/>
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="V43" s="68">
+        <f t="shared" si="8"/>
+        <v>0.97499999999999998</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="K13:L13"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="K23:L23"/>
     <mergeCell ref="K12:L12"/>
     <mergeCell ref="K1:L1"/>
     <mergeCell ref="K2:L2"/>
@@ -13876,28 +14549,6 @@
     <mergeCell ref="K9:L9"/>
     <mergeCell ref="K10:L10"/>
     <mergeCell ref="K11:L11"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="K13:L13"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Agregar junio al dashboard
</commit_message>
<xml_diff>
--- a/Dashboard.xlsx
+++ b/Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauricio\Desktop\NUEVO\DashboardMedico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{729B26A0-31D1-4E96-98B4-8F27F0BD3923}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBD7948-C032-41E7-84DD-9A1AB5BF8F42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{1407A859-4935-4127-A91B-F2429559B5A8}"/>
   </bookViews>
@@ -23,7 +23,7 @@
   </definedNames>
   <calcPr calcId="181029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="49">
   <si>
     <t>mes</t>
   </si>
@@ -188,6 +188,9 @@
   <si>
     <t>mayo</t>
   </si>
+  <si>
+    <t>junio</t>
+  </si>
 </sst>
 </file>
 
@@ -238,7 +241,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -305,8 +308,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="32">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -717,12 +732,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -912,6 +945,34 @@
     <xf numFmtId="10" fontId="4" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -922,12 +983,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -10277,7 +10332,359 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{84E442F7-39EA-4DAC-85E9-0D554B59BD1E}" name="TablaDinámica4" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9343E3D3-8E4C-4B20-B961-BB4621992C8B}" name="TablaDinámica7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+  <location ref="I18:J23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="22">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item h="1" x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="11">
+        <item h="1" x="5"/>
+        <item h="1" x="4"/>
+        <item x="0"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="8"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="9"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Suma de % Rendimiento" fld="12" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{931E7B7E-CA9F-465C-B9CA-2A2FFF91B95F}" name="TablaDinámica6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+  <location ref="F18:G23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="22">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item h="1" x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="11">
+        <item h="1" x="5"/>
+        <item h="1" x="4"/>
+        <item x="0"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="8"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="9"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Suma de % Cumplimiento" fld="6" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="6" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E63473CF-27CE-4690-9F1E-A43D9330F8B0}" name="TablaDinámica5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+  <location ref="F11:I16" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="22">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item h="1" x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="11">
+        <item h="1" x="5"/>
+        <item h="1" x="4"/>
+        <item x="0"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="8"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="9"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+  </colItems>
+  <dataFields count="3">
+    <dataField name="Suma de % formulas" fld="14" baseField="0" baseItem="0"/>
+    <dataField name="Suma de % laboratorios" fld="16" baseField="0" baseItem="0"/>
+    <dataField name="Suma de %Ayudas Diagnosticas" fld="18" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="5">
+    <chartFormat chart="6" format="21" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="22" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="23">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="24">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="25" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{84E442F7-39EA-4DAC-85E9-0D554B59BD1E}" name="TablaDinámica4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E3:L8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="22">
     <pivotField axis="axisRow" showAll="0">
@@ -10423,8 +10830,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8798F489-BE3A-43ED-960C-7BA2B41DFF28}" name="TablaDinámica8" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8798F489-BE3A-43ED-960C-7BA2B41DFF28}" name="TablaDinámica8" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
   <location ref="G26:I31" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="22">
     <pivotField axis="axisRow" showAll="0">
@@ -10553,358 +10960,6 @@
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
             <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9343E3D3-8E4C-4B20-B961-BB4621992C8B}" name="TablaDinámica7" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
-  <location ref="I18:J23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="22">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item h="1" x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="11">
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item x="0"/>
-        <item h="1" x="6"/>
-        <item h="1" x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="8"/>
-        <item h="1" x="7"/>
-        <item h="1" x="3"/>
-        <item h="1" x="9"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Suma de % Rendimiento" fld="12" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="5" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{931E7B7E-CA9F-465C-B9CA-2A2FFF91B95F}" name="TablaDinámica6" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
-  <location ref="F18:G23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="22">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item h="1" x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="11">
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item x="0"/>
-        <item h="1" x="6"/>
-        <item h="1" x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="8"/>
-        <item h="1" x="7"/>
-        <item h="1" x="3"/>
-        <item h="1" x="9"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Suma de % Cumplimiento" fld="6" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="6" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E63473CF-27CE-4690-9F1E-A43D9330F8B0}" name="TablaDinámica5" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
-  <location ref="F11:I16" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="22">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item h="1" x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="11">
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item x="0"/>
-        <item h="1" x="6"/>
-        <item h="1" x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="8"/>
-        <item h="1" x="7"/>
-        <item h="1" x="3"/>
-        <item h="1" x="9"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
-  </colItems>
-  <dataFields count="3">
-    <dataField name="Suma de % formulas" fld="14" baseField="0" baseItem="0"/>
-    <dataField name="Suma de % laboratorios" fld="16" baseField="0" baseItem="0"/>
-    <dataField name="Suma de %Ayudas Diagnosticas" fld="18" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="5">
-    <chartFormat chart="6" format="21" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="22" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="23">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="24">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="25" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="2"/>
           </reference>
         </references>
       </pivotArea>
@@ -11284,7 +11339,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4FD4F9-2910-4648-84AF-C941CDDEB3D5}">
-  <dimension ref="A1:V43"/>
+  <dimension ref="A1:V52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="11.42578125" style="60"/>
@@ -11325,10 +11380,10 @@
       <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="71" t="s">
+      <c r="K1" s="81" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="72"/>
+      <c r="L1" s="82"/>
       <c r="M1" s="63" t="s">
         <v>11</v>
       </c>
@@ -11395,10 +11450,10 @@
       <c r="J2" s="11">
         <v>70</v>
       </c>
-      <c r="K2" s="73">
+      <c r="K2" s="74">
         <v>11</v>
       </c>
-      <c r="L2" s="74"/>
+      <c r="L2" s="75"/>
       <c r="M2" s="64">
         <f>J2/I2</f>
         <v>0.86419753086419748</v>
@@ -11457,7 +11512,7 @@
         <v>2</v>
       </c>
       <c r="G3" s="64">
-        <f t="shared" ref="G3:G43" si="1">E3/D3</f>
+        <f t="shared" ref="G3:G52" si="1">E3/D3</f>
         <v>0.8</v>
       </c>
       <c r="H3" s="14">
@@ -11471,44 +11526,44 @@
       <c r="J3" s="16">
         <v>60</v>
       </c>
-      <c r="K3" s="75">
+      <c r="K3" s="83">
         <v>8</v>
       </c>
-      <c r="L3" s="76"/>
+      <c r="L3" s="84"/>
       <c r="M3" s="64">
-        <f t="shared" ref="M3:M43" si="3">J3/I3</f>
+        <f t="shared" ref="M3:M52" si="3">J3/I3</f>
         <v>0.88235294117647056</v>
       </c>
       <c r="N3" s="17">
         <v>55</v>
       </c>
       <c r="O3" s="66">
-        <f t="shared" ref="O3:O43" si="4">N3/J3</f>
+        <f t="shared" ref="O3:O52" si="4">N3/J3</f>
         <v>0.91666666666666663</v>
       </c>
       <c r="P3" s="16">
         <v>4</v>
       </c>
       <c r="Q3" s="66">
-        <f t="shared" ref="Q3:Q43" si="5">P3/J3</f>
+        <f t="shared" ref="Q3:Q52" si="5">P3/J3</f>
         <v>6.6666666666666666E-2</v>
       </c>
       <c r="R3" s="16">
         <v>2</v>
       </c>
       <c r="S3" s="67">
-        <f t="shared" ref="S3:S43" si="6">R3/J3</f>
+        <f t="shared" ref="S3:S52" si="6">R3/J3</f>
         <v>3.3333333333333333E-2</v>
       </c>
       <c r="T3" s="14">
         <v>7</v>
       </c>
       <c r="U3" s="66">
-        <f t="shared" ref="U3:U43" si="7">T3/J3</f>
+        <f t="shared" ref="U3:U52" si="7">T3/J3</f>
         <v>0.11666666666666667</v>
       </c>
       <c r="V3" s="68">
-        <f t="shared" ref="V3:V43" si="8">(1-(T3/J3))</f>
+        <f t="shared" ref="V3:V52" si="8">(1-(T3/J3))</f>
         <v>0.8833333333333333</v>
       </c>
     </row>
@@ -11547,10 +11602,10 @@
       <c r="J4" s="11">
         <v>50</v>
       </c>
-      <c r="K4" s="69">
+      <c r="K4" s="79">
         <v>10</v>
       </c>
-      <c r="L4" s="70"/>
+      <c r="L4" s="80"/>
       <c r="M4" s="64">
         <f t="shared" si="3"/>
         <v>0.83333333333333337</v>
@@ -11623,10 +11678,10 @@
       <c r="J5" s="11">
         <v>18</v>
       </c>
-      <c r="K5" s="69">
+      <c r="K5" s="79">
         <v>3</v>
       </c>
-      <c r="L5" s="70"/>
+      <c r="L5" s="80"/>
       <c r="M5" s="64">
         <f t="shared" si="3"/>
         <v>0.8571428571428571</v>
@@ -11699,10 +11754,10 @@
       <c r="J6" s="20">
         <v>44</v>
       </c>
-      <c r="K6" s="77">
+      <c r="K6" s="85">
         <v>11</v>
       </c>
-      <c r="L6" s="78"/>
+      <c r="L6" s="86"/>
       <c r="M6" s="64">
         <f t="shared" si="3"/>
         <v>0.8</v>
@@ -11775,10 +11830,10 @@
       <c r="J7" s="16">
         <v>10</v>
       </c>
-      <c r="K7" s="75">
+      <c r="K7" s="83">
         <v>1</v>
       </c>
-      <c r="L7" s="76"/>
+      <c r="L7" s="84"/>
       <c r="M7" s="64">
         <f t="shared" si="3"/>
         <v>0.90909090909090906</v>
@@ -11851,10 +11906,10 @@
       <c r="J8" s="27">
         <v>8</v>
       </c>
-      <c r="K8" s="79">
+      <c r="K8" s="87">
         <v>1</v>
       </c>
-      <c r="L8" s="80"/>
+      <c r="L8" s="88"/>
       <c r="M8" s="64">
         <f t="shared" si="3"/>
         <v>0.88888888888888884</v>
@@ -11927,10 +11982,10 @@
       <c r="J9" s="11">
         <v>139</v>
       </c>
-      <c r="K9" s="73">
+      <c r="K9" s="74">
         <v>4</v>
       </c>
-      <c r="L9" s="74"/>
+      <c r="L9" s="75"/>
       <c r="M9" s="64">
         <f t="shared" si="3"/>
         <v>0.97202797202797198</v>
@@ -12003,10 +12058,10 @@
       <c r="J10" s="16">
         <v>112</v>
       </c>
-      <c r="K10" s="75">
+      <c r="K10" s="83">
         <v>2</v>
       </c>
-      <c r="L10" s="76"/>
+      <c r="L10" s="84"/>
       <c r="M10" s="64">
         <f t="shared" si="3"/>
         <v>0.98245614035087714</v>
@@ -12079,10 +12134,10 @@
       <c r="J11" s="11">
         <v>77</v>
       </c>
-      <c r="K11" s="69">
+      <c r="K11" s="79">
         <v>1</v>
       </c>
-      <c r="L11" s="70"/>
+      <c r="L11" s="80"/>
       <c r="M11" s="64">
         <f t="shared" si="3"/>
         <v>0.98717948717948723</v>
@@ -12155,10 +12210,10 @@
       <c r="J12" s="11">
         <v>61</v>
       </c>
-      <c r="K12" s="69">
+      <c r="K12" s="79">
         <v>4</v>
       </c>
-      <c r="L12" s="70"/>
+      <c r="L12" s="80"/>
       <c r="M12" s="64">
         <f t="shared" si="3"/>
         <v>0.93846153846153846</v>
@@ -12231,10 +12286,10 @@
       <c r="J13" s="20">
         <v>64</v>
       </c>
-      <c r="K13" s="77">
+      <c r="K13" s="85">
         <v>1</v>
       </c>
-      <c r="L13" s="78"/>
+      <c r="L13" s="86"/>
       <c r="M13" s="64">
         <f t="shared" si="3"/>
         <v>0.98461538461538467</v>
@@ -12307,10 +12362,10 @@
       <c r="J14" s="16">
         <v>21</v>
       </c>
-      <c r="K14" s="75">
+      <c r="K14" s="83">
         <v>1</v>
       </c>
-      <c r="L14" s="76"/>
+      <c r="L14" s="84"/>
       <c r="M14" s="64">
         <f t="shared" si="3"/>
         <v>0.95454545454545459</v>
@@ -12382,10 +12437,10 @@
       <c r="J15" s="34">
         <v>28</v>
       </c>
-      <c r="K15" s="81">
+      <c r="K15" s="89">
         <v>0</v>
       </c>
-      <c r="L15" s="82"/>
+      <c r="L15" s="90"/>
       <c r="M15" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -12458,10 +12513,10 @@
       <c r="J16" s="40">
         <v>23</v>
       </c>
-      <c r="K16" s="83">
+      <c r="K16" s="91">
         <v>1</v>
       </c>
-      <c r="L16" s="84"/>
+      <c r="L16" s="92"/>
       <c r="M16" s="64">
         <f t="shared" si="3"/>
         <v>0.95833333333333337</v>
@@ -12534,10 +12589,10 @@
       <c r="J17" s="11">
         <v>164</v>
       </c>
-      <c r="K17" s="73">
+      <c r="K17" s="74">
         <v>2</v>
       </c>
-      <c r="L17" s="74"/>
+      <c r="L17" s="75"/>
       <c r="M17" s="64">
         <f t="shared" si="3"/>
         <v>0.98795180722891562</v>
@@ -12610,10 +12665,10 @@
       <c r="J18" s="16">
         <v>133</v>
       </c>
-      <c r="K18" s="75">
+      <c r="K18" s="83">
         <v>2</v>
       </c>
-      <c r="L18" s="76"/>
+      <c r="L18" s="84"/>
       <c r="M18" s="64">
         <f t="shared" si="3"/>
         <v>0.98518518518518516</v>
@@ -12686,10 +12741,10 @@
       <c r="J19" s="11">
         <v>111</v>
       </c>
-      <c r="K19" s="69">
+      <c r="K19" s="79">
         <v>1</v>
       </c>
-      <c r="L19" s="70"/>
+      <c r="L19" s="80"/>
       <c r="M19" s="64">
         <f t="shared" si="3"/>
         <v>0.9910714285714286</v>
@@ -12762,10 +12817,10 @@
       <c r="J20" s="11">
         <v>76</v>
       </c>
-      <c r="K20" s="69">
+      <c r="K20" s="79">
         <v>1</v>
       </c>
-      <c r="L20" s="70"/>
+      <c r="L20" s="80"/>
       <c r="M20" s="64">
         <f t="shared" si="3"/>
         <v>0.98701298701298701</v>
@@ -12837,10 +12892,10 @@
       <c r="J21" s="11">
         <v>43</v>
       </c>
-      <c r="K21" s="69">
+      <c r="K21" s="79">
         <v>2</v>
       </c>
-      <c r="L21" s="70"/>
+      <c r="L21" s="80"/>
       <c r="M21" s="64">
         <f t="shared" si="3"/>
         <v>0.9555555555555556</v>
@@ -12913,10 +12968,10 @@
       <c r="J22" s="20">
         <v>86</v>
       </c>
-      <c r="K22" s="77">
+      <c r="K22" s="85">
         <v>1</v>
       </c>
-      <c r="L22" s="78"/>
+      <c r="L22" s="86"/>
       <c r="M22" s="64">
         <f t="shared" si="3"/>
         <v>0.9885057471264368</v>
@@ -12989,10 +13044,10 @@
       <c r="J23" s="16">
         <v>26</v>
       </c>
-      <c r="K23" s="75">
+      <c r="K23" s="83">
         <v>1</v>
       </c>
-      <c r="L23" s="76"/>
+      <c r="L23" s="84"/>
       <c r="M23" s="64">
         <f t="shared" si="3"/>
         <v>0.96296296296296291</v>
@@ -13064,10 +13119,10 @@
       <c r="J24" s="34">
         <v>30</v>
       </c>
-      <c r="K24" s="81">
+      <c r="K24" s="89">
         <v>0</v>
       </c>
-      <c r="L24" s="82"/>
+      <c r="L24" s="90"/>
       <c r="M24" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -13140,10 +13195,10 @@
       <c r="J25" s="49">
         <v>43</v>
       </c>
-      <c r="K25" s="85">
+      <c r="K25" s="93">
         <v>2</v>
       </c>
-      <c r="L25" s="86"/>
+      <c r="L25" s="94"/>
       <c r="M25" s="64">
         <f t="shared" si="3"/>
         <v>0.9555555555555556</v>
@@ -13215,11 +13270,11 @@
       <c r="J26" s="56">
         <v>143</v>
       </c>
-      <c r="K26" s="87">
+      <c r="K26" s="95">
         <f>I26-J26</f>
         <v>6</v>
       </c>
-      <c r="L26" s="88"/>
+      <c r="L26" s="96"/>
       <c r="M26" s="64">
         <f t="shared" si="3"/>
         <v>0.95973154362416102</v>
@@ -13291,11 +13346,11 @@
       <c r="J27" s="16">
         <v>74</v>
       </c>
-      <c r="K27" s="73">
+      <c r="K27" s="74">
         <f>I27-J27</f>
         <v>1</v>
       </c>
-      <c r="L27" s="74"/>
+      <c r="L27" s="75"/>
       <c r="M27" s="64">
         <f t="shared" si="3"/>
         <v>0.98666666666666669</v>
@@ -13367,11 +13422,11 @@
       <c r="J28" s="11">
         <v>83</v>
       </c>
-      <c r="K28" s="73">
+      <c r="K28" s="74">
         <f t="shared" ref="K28:K29" si="20">I28-J28</f>
         <v>0</v>
       </c>
-      <c r="L28" s="74"/>
+      <c r="L28" s="75"/>
       <c r="M28" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -13443,11 +13498,11 @@
       <c r="J29" s="11">
         <v>79</v>
       </c>
-      <c r="K29" s="73">
+      <c r="K29" s="74">
         <f t="shared" si="20"/>
         <v>3</v>
       </c>
-      <c r="L29" s="74"/>
+      <c r="L29" s="75"/>
       <c r="M29" s="64">
         <f t="shared" si="3"/>
         <v>0.96341463414634143</v>
@@ -13519,11 +13574,11 @@
       <c r="J30" s="11">
         <v>93</v>
       </c>
-      <c r="K30" s="73">
+      <c r="K30" s="74">
         <f>I30-J30</f>
         <v>0</v>
       </c>
-      <c r="L30" s="74"/>
+      <c r="L30" s="75"/>
       <c r="M30" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -13595,11 +13650,11 @@
       <c r="J31" s="20">
         <v>78</v>
       </c>
-      <c r="K31" s="73">
+      <c r="K31" s="74">
         <f>I31-J31</f>
         <v>1</v>
       </c>
-      <c r="L31" s="74"/>
+      <c r="L31" s="75"/>
       <c r="M31" s="64">
         <f t="shared" si="3"/>
         <v>0.98734177215189878</v>
@@ -13671,11 +13726,11 @@
       <c r="J32" s="16">
         <v>33</v>
       </c>
-      <c r="K32" s="73">
+      <c r="K32" s="74">
         <f t="shared" ref="K32:K33" si="22">I32-J32</f>
         <v>0</v>
       </c>
-      <c r="L32" s="74"/>
+      <c r="L32" s="75"/>
       <c r="M32" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -13747,11 +13802,11 @@
       <c r="J33" s="34">
         <v>28</v>
       </c>
-      <c r="K33" s="73">
+      <c r="K33" s="74">
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
-      <c r="L33" s="74"/>
+      <c r="L33" s="75"/>
       <c r="M33" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -13823,11 +13878,11 @@
       <c r="J34" s="49">
         <v>35</v>
       </c>
-      <c r="K34" s="73">
+      <c r="K34" s="74">
         <f>I34-J34</f>
         <v>2</v>
       </c>
-      <c r="L34" s="74"/>
+      <c r="L34" s="75"/>
       <c r="M34" s="64">
         <f t="shared" si="3"/>
         <v>0.94594594594594594</v>
@@ -13897,9 +13952,10 @@
       <c r="J35">
         <v>134</v>
       </c>
-      <c r="K35">
+      <c r="K35" s="76">
         <v>27</v>
       </c>
+      <c r="L35" s="76"/>
       <c r="M35" s="64">
         <f t="shared" si="3"/>
         <v>0.83229813664596275</v>
@@ -13969,9 +14025,10 @@
       <c r="J36">
         <v>118</v>
       </c>
-      <c r="K36">
+      <c r="K36" s="77">
         <v>33</v>
       </c>
+      <c r="L36" s="77"/>
       <c r="M36" s="64">
         <f t="shared" si="3"/>
         <v>0.7814569536423841</v>
@@ -14041,9 +14098,10 @@
       <c r="J37">
         <v>86</v>
       </c>
-      <c r="K37">
+      <c r="K37" s="77">
         <v>40</v>
       </c>
+      <c r="L37" s="77"/>
       <c r="M37" s="64">
         <f t="shared" si="3"/>
         <v>0.68253968253968256</v>
@@ -14113,9 +14171,10 @@
       <c r="J38">
         <v>91</v>
       </c>
-      <c r="K38">
+      <c r="K38" s="77">
         <v>35</v>
       </c>
+      <c r="L38" s="77"/>
       <c r="M38" s="64">
         <f t="shared" si="3"/>
         <v>0.72222222222222221</v>
@@ -14185,9 +14244,10 @@
       <c r="J39">
         <v>92</v>
       </c>
-      <c r="K39">
+      <c r="K39" s="77">
         <v>38</v>
       </c>
+      <c r="L39" s="77"/>
       <c r="M39" s="64">
         <f t="shared" si="3"/>
         <v>0.70769230769230773</v>
@@ -14257,9 +14317,10 @@
       <c r="J40">
         <v>53</v>
       </c>
-      <c r="K40">
+      <c r="K40" s="77">
         <v>23</v>
       </c>
+      <c r="L40" s="77"/>
       <c r="M40" s="64">
         <f t="shared" si="3"/>
         <v>0.69736842105263153</v>
@@ -14329,9 +14390,10 @@
       <c r="J41">
         <v>29</v>
       </c>
-      <c r="K41">
+      <c r="K41" s="77">
         <v>5</v>
       </c>
+      <c r="L41" s="77"/>
       <c r="M41" s="64">
         <f t="shared" si="3"/>
         <v>0.8529411764705882</v>
@@ -14401,9 +14463,10 @@
       <c r="J42">
         <v>22</v>
       </c>
-      <c r="K42">
+      <c r="K42" s="77">
         <v>7</v>
       </c>
+      <c r="L42" s="77"/>
       <c r="M42" s="64">
         <f t="shared" si="3"/>
         <v>0.75862068965517238</v>
@@ -14473,9 +14536,10 @@
       <c r="J43">
         <v>40</v>
       </c>
-      <c r="K43">
+      <c r="K43" s="78">
         <v>20</v>
       </c>
+      <c r="L43" s="78"/>
       <c r="M43" s="64">
         <f t="shared" si="3"/>
         <v>0.66666666666666663</v>
@@ -14513,8 +14577,692 @@
         <v>0.97499999999999998</v>
       </c>
     </row>
+    <row r="44" spans="1:22" s="69" customFormat="1" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="69" t="s">
+        <v>48</v>
+      </c>
+      <c r="B44" t="s">
+        <v>22</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D44" s="9">
+        <v>18</v>
+      </c>
+      <c r="E44" s="10">
+        <v>15</v>
+      </c>
+      <c r="F44" s="11">
+        <f>D44-E44</f>
+        <v>3</v>
+      </c>
+      <c r="G44" s="64">
+        <f t="shared" si="1"/>
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="H44" s="9">
+        <f>E44*4*3</f>
+        <v>180</v>
+      </c>
+      <c r="I44" s="11">
+        <f>J44+K44</f>
+        <v>126</v>
+      </c>
+      <c r="J44" s="70">
+        <v>98</v>
+      </c>
+      <c r="K44" s="74">
+        <v>28</v>
+      </c>
+      <c r="L44" s="75"/>
+      <c r="M44" s="64">
+        <f t="shared" si="3"/>
+        <v>0.77777777777777779</v>
+      </c>
+      <c r="N44" s="12">
+        <v>72</v>
+      </c>
+      <c r="O44" s="66">
+        <f t="shared" si="4"/>
+        <v>0.73469387755102045</v>
+      </c>
+      <c r="P44" s="11">
+        <v>35</v>
+      </c>
+      <c r="Q44" s="66">
+        <f t="shared" si="5"/>
+        <v>0.35714285714285715</v>
+      </c>
+      <c r="R44" s="11">
+        <v>11</v>
+      </c>
+      <c r="S44" s="67">
+        <f t="shared" si="6"/>
+        <v>0.11224489795918367</v>
+      </c>
+      <c r="T44" s="9">
+        <v>19</v>
+      </c>
+      <c r="U44" s="66">
+        <f t="shared" si="7"/>
+        <v>0.19387755102040816</v>
+      </c>
+      <c r="V44" s="68">
+        <f t="shared" si="8"/>
+        <v>0.80612244897959184</v>
+      </c>
+    </row>
+    <row r="45" spans="1:22" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="69" t="s">
+        <v>48</v>
+      </c>
+      <c r="B45" t="s">
+        <v>22</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D45" s="14">
+        <v>18</v>
+      </c>
+      <c r="E45" s="15">
+        <v>16</v>
+      </c>
+      <c r="F45" s="11">
+        <f t="shared" ref="F45:F48" si="23">D45-E45</f>
+        <v>2</v>
+      </c>
+      <c r="G45" s="64">
+        <f t="shared" si="1"/>
+        <v>0.88888888888888884</v>
+      </c>
+      <c r="H45" s="14">
+        <f>E45*4*2</f>
+        <v>128</v>
+      </c>
+      <c r="I45" s="11">
+        <f>J45+K45</f>
+        <v>134</v>
+      </c>
+      <c r="J45" s="70">
+        <v>101</v>
+      </c>
+      <c r="K45" s="74">
+        <v>33</v>
+      </c>
+      <c r="L45" s="75"/>
+      <c r="M45" s="64">
+        <f t="shared" si="3"/>
+        <v>0.75373134328358204</v>
+      </c>
+      <c r="N45" s="17">
+        <v>124</v>
+      </c>
+      <c r="O45" s="66">
+        <f t="shared" si="4"/>
+        <v>1.2277227722772277</v>
+      </c>
+      <c r="P45" s="16">
+        <v>67</v>
+      </c>
+      <c r="Q45" s="66">
+        <f t="shared" si="5"/>
+        <v>0.6633663366336634</v>
+      </c>
+      <c r="R45" s="16">
+        <v>11</v>
+      </c>
+      <c r="S45" s="67">
+        <f t="shared" si="6"/>
+        <v>0.10891089108910891</v>
+      </c>
+      <c r="T45" s="14">
+        <v>19</v>
+      </c>
+      <c r="U45" s="66">
+        <f t="shared" si="7"/>
+        <v>0.18811881188118812</v>
+      </c>
+      <c r="V45" s="68">
+        <f t="shared" si="8"/>
+        <v>0.81188118811881194</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="69" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" t="s">
+        <v>22</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D46" s="9">
+        <v>18</v>
+      </c>
+      <c r="E46" s="10">
+        <v>17</v>
+      </c>
+      <c r="F46" s="11">
+        <f t="shared" si="23"/>
+        <v>1</v>
+      </c>
+      <c r="G46" s="64">
+        <f t="shared" si="1"/>
+        <v>0.94444444444444442</v>
+      </c>
+      <c r="H46" s="9">
+        <f>E46*4*2</f>
+        <v>136</v>
+      </c>
+      <c r="I46" s="11">
+        <f>J46+K46</f>
+        <v>102</v>
+      </c>
+      <c r="J46" s="70">
+        <v>83</v>
+      </c>
+      <c r="K46" s="74">
+        <v>19</v>
+      </c>
+      <c r="L46" s="75"/>
+      <c r="M46" s="64">
+        <f t="shared" si="3"/>
+        <v>0.81372549019607843</v>
+      </c>
+      <c r="N46" s="12">
+        <v>165</v>
+      </c>
+      <c r="O46" s="66">
+        <f t="shared" si="4"/>
+        <v>1.9879518072289157</v>
+      </c>
+      <c r="P46" s="11">
+        <v>31</v>
+      </c>
+      <c r="Q46" s="66">
+        <f t="shared" si="5"/>
+        <v>0.37349397590361444</v>
+      </c>
+      <c r="R46" s="11">
+        <v>16</v>
+      </c>
+      <c r="S46" s="67">
+        <f t="shared" si="6"/>
+        <v>0.19277108433734941</v>
+      </c>
+      <c r="T46" s="9">
+        <v>13</v>
+      </c>
+      <c r="U46" s="66">
+        <f t="shared" si="7"/>
+        <v>0.15662650602409639</v>
+      </c>
+      <c r="V46" s="68">
+        <f t="shared" si="8"/>
+        <v>0.84337349397590367</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="69" t="s">
+        <v>48</v>
+      </c>
+      <c r="B47" t="s">
+        <v>22</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D47" s="9">
+        <v>18</v>
+      </c>
+      <c r="E47" s="10">
+        <v>14</v>
+      </c>
+      <c r="F47" s="11">
+        <f t="shared" si="23"/>
+        <v>4</v>
+      </c>
+      <c r="G47" s="64">
+        <f t="shared" si="1"/>
+        <v>0.77777777777777779</v>
+      </c>
+      <c r="H47" s="9">
+        <f>E47*4*2</f>
+        <v>112</v>
+      </c>
+      <c r="I47" s="11">
+        <f t="shared" ref="I47:I52" si="24">J47+K47</f>
+        <v>86</v>
+      </c>
+      <c r="J47" s="70">
+        <v>65</v>
+      </c>
+      <c r="K47" s="74">
+        <v>21</v>
+      </c>
+      <c r="L47" s="75"/>
+      <c r="M47" s="64">
+        <f t="shared" si="3"/>
+        <v>0.7558139534883721</v>
+      </c>
+      <c r="N47" s="12">
+        <v>134</v>
+      </c>
+      <c r="O47" s="66">
+        <f t="shared" si="4"/>
+        <v>2.0615384615384613</v>
+      </c>
+      <c r="P47" s="11">
+        <v>13</v>
+      </c>
+      <c r="Q47" s="66">
+        <f t="shared" si="5"/>
+        <v>0.2</v>
+      </c>
+      <c r="R47" s="11">
+        <v>4</v>
+      </c>
+      <c r="S47" s="67">
+        <f t="shared" si="6"/>
+        <v>6.1538461538461542E-2</v>
+      </c>
+      <c r="T47" s="9">
+        <v>10</v>
+      </c>
+      <c r="U47" s="66">
+        <f t="shared" si="7"/>
+        <v>0.15384615384615385</v>
+      </c>
+      <c r="V47" s="68">
+        <f t="shared" si="8"/>
+        <v>0.84615384615384615</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="69" t="s">
+        <v>48</v>
+      </c>
+      <c r="B48" t="s">
+        <v>35</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D48" s="9">
+        <v>18</v>
+      </c>
+      <c r="E48" s="10">
+        <v>16</v>
+      </c>
+      <c r="F48" s="11">
+        <f t="shared" si="23"/>
+        <v>2</v>
+      </c>
+      <c r="G48" s="64">
+        <f t="shared" si="1"/>
+        <v>0.88888888888888884</v>
+      </c>
+      <c r="H48" s="9">
+        <f>E48*3*2</f>
+        <v>96</v>
+      </c>
+      <c r="I48" s="11">
+        <f t="shared" si="24"/>
+        <v>116</v>
+      </c>
+      <c r="J48" s="70">
+        <v>93</v>
+      </c>
+      <c r="K48" s="74">
+        <v>23</v>
+      </c>
+      <c r="L48" s="75"/>
+      <c r="M48" s="64">
+        <f t="shared" si="3"/>
+        <v>0.80172413793103448</v>
+      </c>
+      <c r="N48" s="12">
+        <v>147</v>
+      </c>
+      <c r="O48" s="66">
+        <f t="shared" si="4"/>
+        <v>1.5806451612903225</v>
+      </c>
+      <c r="P48" s="11">
+        <v>113</v>
+      </c>
+      <c r="Q48" s="66">
+        <f t="shared" si="5"/>
+        <v>1.2150537634408602</v>
+      </c>
+      <c r="R48" s="11">
+        <v>40</v>
+      </c>
+      <c r="S48" s="67">
+        <f t="shared" si="6"/>
+        <v>0.43010752688172044</v>
+      </c>
+      <c r="T48" s="9">
+        <v>15</v>
+      </c>
+      <c r="U48" s="66">
+        <f t="shared" si="7"/>
+        <v>0.16129032258064516</v>
+      </c>
+      <c r="V48" s="68">
+        <f t="shared" si="8"/>
+        <v>0.83870967741935487</v>
+      </c>
+    </row>
+    <row r="49" spans="1:22" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="69" t="s">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>27</v>
+      </c>
+      <c r="C49" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D49" s="18">
+        <v>18</v>
+      </c>
+      <c r="E49" s="19">
+        <v>15</v>
+      </c>
+      <c r="F49" s="20">
+        <f>D49-E49</f>
+        <v>3</v>
+      </c>
+      <c r="G49" s="64">
+        <f t="shared" si="1"/>
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="H49" s="18">
+        <f>E49*8*2</f>
+        <v>240</v>
+      </c>
+      <c r="I49" s="11">
+        <f t="shared" si="24"/>
+        <v>62</v>
+      </c>
+      <c r="J49" s="71">
+        <v>48</v>
+      </c>
+      <c r="K49" s="74">
+        <v>14</v>
+      </c>
+      <c r="L49" s="75"/>
+      <c r="M49" s="64">
+        <f t="shared" si="3"/>
+        <v>0.77419354838709675</v>
+      </c>
+      <c r="N49" s="21">
+        <v>0</v>
+      </c>
+      <c r="O49" s="66">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="P49" s="20">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="66">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R49" s="20">
+        <v>7</v>
+      </c>
+      <c r="S49" s="67">
+        <f t="shared" si="6"/>
+        <v>0.14583333333333334</v>
+      </c>
+      <c r="T49" s="18">
+        <v>14</v>
+      </c>
+      <c r="U49" s="66">
+        <f t="shared" si="7"/>
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="V49" s="68">
+        <f t="shared" si="8"/>
+        <v>0.70833333333333326</v>
+      </c>
+    </row>
+    <row r="50" spans="1:22" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="69" t="s">
+        <v>48</v>
+      </c>
+      <c r="B50" t="s">
+        <v>27</v>
+      </c>
+      <c r="C50" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="D50" s="14">
+        <v>18</v>
+      </c>
+      <c r="E50" s="15">
+        <v>13</v>
+      </c>
+      <c r="F50" s="20">
+        <f t="shared" ref="F50:F51" si="25">D50-E50</f>
+        <v>5</v>
+      </c>
+      <c r="G50" s="64">
+        <f t="shared" si="1"/>
+        <v>0.72222222222222221</v>
+      </c>
+      <c r="H50" s="14">
+        <f>E50*4*2</f>
+        <v>104</v>
+      </c>
+      <c r="I50" s="11">
+        <f t="shared" si="24"/>
+        <v>34</v>
+      </c>
+      <c r="J50" s="70">
+        <v>26</v>
+      </c>
+      <c r="K50" s="74">
+        <v>8</v>
+      </c>
+      <c r="L50" s="75"/>
+      <c r="M50" s="64">
+        <f t="shared" si="3"/>
+        <v>0.76470588235294112</v>
+      </c>
+      <c r="N50" s="17">
+        <v>2</v>
+      </c>
+      <c r="O50" s="66">
+        <f t="shared" si="4"/>
+        <v>7.6923076923076927E-2</v>
+      </c>
+      <c r="P50" s="16">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="66">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R50" s="16">
+        <v>7</v>
+      </c>
+      <c r="S50" s="67">
+        <f t="shared" si="6"/>
+        <v>0.26923076923076922</v>
+      </c>
+      <c r="T50" s="14">
+        <v>9</v>
+      </c>
+      <c r="U50" s="66">
+        <f t="shared" si="7"/>
+        <v>0.34615384615384615</v>
+      </c>
+      <c r="V50" s="68">
+        <f t="shared" si="8"/>
+        <v>0.65384615384615385</v>
+      </c>
+    </row>
+    <row r="51" spans="1:22" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="69" t="s">
+        <v>48</v>
+      </c>
+      <c r="B51" t="s">
+        <v>27</v>
+      </c>
+      <c r="C51" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="D51" s="32">
+        <v>18</v>
+      </c>
+      <c r="E51" s="33">
+        <v>10</v>
+      </c>
+      <c r="F51" s="20">
+        <f t="shared" si="25"/>
+        <v>8</v>
+      </c>
+      <c r="G51" s="64">
+        <f t="shared" si="1"/>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="H51" s="32">
+        <f>E51*4*2</f>
+        <v>80</v>
+      </c>
+      <c r="I51" s="11">
+        <f t="shared" si="24"/>
+        <v>31</v>
+      </c>
+      <c r="J51" s="72">
+        <v>21</v>
+      </c>
+      <c r="K51" s="74">
+        <v>10</v>
+      </c>
+      <c r="L51" s="75"/>
+      <c r="M51" s="64">
+        <f t="shared" si="3"/>
+        <v>0.67741935483870963</v>
+      </c>
+      <c r="N51" s="35">
+        <v>2</v>
+      </c>
+      <c r="O51" s="66">
+        <f t="shared" si="4"/>
+        <v>9.5238095238095233E-2</v>
+      </c>
+      <c r="P51" s="34">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="66">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R51" s="34">
+        <v>2</v>
+      </c>
+      <c r="S51" s="67">
+        <f t="shared" si="6"/>
+        <v>9.5238095238095233E-2</v>
+      </c>
+      <c r="T51" s="32">
+        <v>4</v>
+      </c>
+      <c r="U51" s="66">
+        <f t="shared" si="7"/>
+        <v>0.19047619047619047</v>
+      </c>
+      <c r="V51" s="68">
+        <f t="shared" si="8"/>
+        <v>0.80952380952380953</v>
+      </c>
+    </row>
+    <row r="52" spans="1:22" ht="46.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="69" t="s">
+        <v>48</v>
+      </c>
+      <c r="B52" t="s">
+        <v>30</v>
+      </c>
+      <c r="C52" s="44" t="s">
+        <v>31</v>
+      </c>
+      <c r="D52" s="45">
+        <v>16</v>
+      </c>
+      <c r="E52" s="46">
+        <v>12</v>
+      </c>
+      <c r="F52" s="47">
+        <f>D52-E52</f>
+        <v>4</v>
+      </c>
+      <c r="G52" s="64">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
+      <c r="H52" s="45">
+        <f>E52*4*2</f>
+        <v>96</v>
+      </c>
+      <c r="I52" s="11">
+        <f t="shared" si="24"/>
+        <v>65</v>
+      </c>
+      <c r="J52" s="73">
+        <v>43</v>
+      </c>
+      <c r="K52" s="74">
+        <v>22</v>
+      </c>
+      <c r="L52" s="75"/>
+      <c r="M52" s="64">
+        <f t="shared" si="3"/>
+        <v>0.66153846153846152</v>
+      </c>
+      <c r="N52" s="50">
+        <v>0</v>
+      </c>
+      <c r="O52" s="66">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="P52" s="49">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="66">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R52" s="49">
+        <v>0</v>
+      </c>
+      <c r="S52" s="67">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="T52" s="51">
+        <v>1</v>
+      </c>
+      <c r="U52" s="66">
+        <f t="shared" si="7"/>
+        <v>2.3255813953488372E-2</v>
+      </c>
+      <c r="V52" s="68">
+        <f t="shared" si="8"/>
+        <v>0.97674418604651159</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="52">
     <mergeCell ref="K31:L31"/>
     <mergeCell ref="K32:L32"/>
     <mergeCell ref="K33:L33"/>
@@ -14525,18 +15273,18 @@
     <mergeCell ref="K28:L28"/>
     <mergeCell ref="K29:L29"/>
     <mergeCell ref="K30:L30"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="K13:L13"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="K23:L23"/>
     <mergeCell ref="K14:L14"/>
     <mergeCell ref="K15:L15"/>
     <mergeCell ref="K16:L16"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="K18:L18"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="K47:L47"/>
+    <mergeCell ref="K48:L48"/>
     <mergeCell ref="K12:L12"/>
     <mergeCell ref="K1:L1"/>
     <mergeCell ref="K2:L2"/>
@@ -14549,6 +15297,24 @@
     <mergeCell ref="K9:L9"/>
     <mergeCell ref="K10:L10"/>
     <mergeCell ref="K11:L11"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="K13:L13"/>
+    <mergeCell ref="K49:L49"/>
+    <mergeCell ref="K50:L50"/>
+    <mergeCell ref="K51:L51"/>
+    <mergeCell ref="K52:L52"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="K36:L36"/>
+    <mergeCell ref="K37:L37"/>
+    <mergeCell ref="K38:L38"/>
+    <mergeCell ref="K39:L39"/>
+    <mergeCell ref="K40:L40"/>
+    <mergeCell ref="K41:L41"/>
+    <mergeCell ref="K42:L42"/>
+    <mergeCell ref="K43:L43"/>
+    <mergeCell ref="K44:L44"/>
+    <mergeCell ref="K45:L45"/>
+    <mergeCell ref="K46:L46"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Agregar julio al dashboard
</commit_message>
<xml_diff>
--- a/Dashboard.xlsx
+++ b/Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauricio\Desktop\NUEVO\DashboardMedico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBD7948-C032-41E7-84DD-9A1AB5BF8F42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0ED85C7-1BD5-404E-9B3B-6155BA643C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{1407A859-4935-4127-A91B-F2429559B5A8}"/>
   </bookViews>
@@ -23,7 +23,7 @@
   </definedNames>
   <calcPr calcId="181029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId4"/>
+    <pivotCache cacheId="2" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="50">
   <si>
     <t>mes</t>
   </si>
@@ -190,6 +190,9 @@
   </si>
   <si>
     <t>junio</t>
+  </si>
+  <si>
+    <t>julio</t>
   </si>
 </sst>
 </file>
@@ -964,31 +967,22 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -997,10 +991,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1015,17 +1009,26 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1052,8 +1055,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF00CC00"/>
       <color rgb="FF559C00"/>
-      <color rgb="FF00CC00"/>
     </mruColors>
   </colors>
   <extLst>
@@ -10332,205 +10335,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9343E3D3-8E4C-4B20-B961-BB4621992C8B}" name="TablaDinámica7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
-  <location ref="I18:J23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="22">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item h="1" x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="11">
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item x="0"/>
-        <item h="1" x="6"/>
-        <item h="1" x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="8"/>
-        <item h="1" x="7"/>
-        <item h="1" x="3"/>
-        <item h="1" x="9"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Suma de % Rendimiento" fld="12" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="5" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{931E7B7E-CA9F-465C-B9CA-2A2FFF91B95F}" name="TablaDinámica6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
-  <location ref="F18:G23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="22">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item h="1" x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="11">
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item x="0"/>
-        <item h="1" x="6"/>
-        <item h="1" x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="8"/>
-        <item h="1" x="7"/>
-        <item h="1" x="3"/>
-        <item h="1" x="9"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Suma de % Cumplimiento" fld="6" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="6" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E63473CF-27CE-4690-9F1E-A43D9330F8B0}" name="TablaDinámica5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E63473CF-27CE-4690-9F1E-A43D9330F8B0}" name="TablaDinámica5" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
   <location ref="F11:I16" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="22">
     <pivotField axis="axisRow" showAll="0">
@@ -10683,8 +10488,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{84E442F7-39EA-4DAC-85E9-0D554B59BD1E}" name="TablaDinámica4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{84E442F7-39EA-4DAC-85E9-0D554B59BD1E}" name="TablaDinámica4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E3:L8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="22">
     <pivotField axis="axisRow" showAll="0">
@@ -10830,8 +10635,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8798F489-BE3A-43ED-960C-7BA2B41DFF28}" name="TablaDinámica8" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8798F489-BE3A-43ED-960C-7BA2B41DFF28}" name="TablaDinámica8" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
   <location ref="G26:I31" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="22">
     <pivotField axis="axisRow" showAll="0">
@@ -10960,6 +10765,204 @@
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
             <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9343E3D3-8E4C-4B20-B961-BB4621992C8B}" name="TablaDinámica7" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+  <location ref="I18:J23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="22">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item h="1" x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="11">
+        <item h="1" x="5"/>
+        <item h="1" x="4"/>
+        <item x="0"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="8"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="9"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Suma de % Rendimiento" fld="12" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{931E7B7E-CA9F-465C-B9CA-2A2FFF91B95F}" name="TablaDinámica6" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="3">
+  <location ref="F18:G23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="22">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item h="1" x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="11">
+        <item h="1" x="5"/>
+        <item h="1" x="4"/>
+        <item x="0"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="8"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="9"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Suma de % Cumplimiento" fld="6" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="6" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
           </reference>
         </references>
       </pivotArea>
@@ -11339,7 +11342,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4FD4F9-2910-4648-84AF-C941CDDEB3D5}">
-  <dimension ref="A1:V52"/>
+  <dimension ref="A1:V61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="11.42578125" style="60"/>
@@ -11380,10 +11383,10 @@
       <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="81" t="s">
+      <c r="K1" s="90" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="82"/>
+      <c r="L1" s="91"/>
       <c r="M1" s="63" t="s">
         <v>11</v>
       </c>
@@ -11512,7 +11515,7 @@
         <v>2</v>
       </c>
       <c r="G3" s="64">
-        <f t="shared" ref="G3:G52" si="1">E3/D3</f>
+        <f t="shared" ref="G3:G61" si="1">E3/D3</f>
         <v>0.8</v>
       </c>
       <c r="H3" s="14">
@@ -11526,44 +11529,44 @@
       <c r="J3" s="16">
         <v>60</v>
       </c>
-      <c r="K3" s="83">
+      <c r="K3" s="84">
         <v>8</v>
       </c>
-      <c r="L3" s="84"/>
+      <c r="L3" s="85"/>
       <c r="M3" s="64">
-        <f t="shared" ref="M3:M52" si="3">J3/I3</f>
+        <f t="shared" ref="M3:M61" si="3">J3/I3</f>
         <v>0.88235294117647056</v>
       </c>
       <c r="N3" s="17">
         <v>55</v>
       </c>
       <c r="O3" s="66">
-        <f t="shared" ref="O3:O52" si="4">N3/J3</f>
+        <f t="shared" ref="O3:O61" si="4">N3/J3</f>
         <v>0.91666666666666663</v>
       </c>
       <c r="P3" s="16">
         <v>4</v>
       </c>
       <c r="Q3" s="66">
-        <f t="shared" ref="Q3:Q52" si="5">P3/J3</f>
+        <f t="shared" ref="Q3:Q61" si="5">P3/J3</f>
         <v>6.6666666666666666E-2</v>
       </c>
       <c r="R3" s="16">
         <v>2</v>
       </c>
       <c r="S3" s="67">
-        <f t="shared" ref="S3:S52" si="6">R3/J3</f>
+        <f t="shared" ref="S3:S61" si="6">R3/J3</f>
         <v>3.3333333333333333E-2</v>
       </c>
       <c r="T3" s="14">
         <v>7</v>
       </c>
       <c r="U3" s="66">
-        <f t="shared" ref="U3:U52" si="7">T3/J3</f>
+        <f t="shared" ref="U3:U61" si="7">T3/J3</f>
         <v>0.11666666666666667</v>
       </c>
       <c r="V3" s="68">
-        <f t="shared" ref="V3:V52" si="8">(1-(T3/J3))</f>
+        <f t="shared" ref="V3:V61" si="8">(1-(T3/J3))</f>
         <v>0.8833333333333333</v>
       </c>
     </row>
@@ -11602,10 +11605,10 @@
       <c r="J4" s="11">
         <v>50</v>
       </c>
-      <c r="K4" s="79">
+      <c r="K4" s="80">
         <v>10</v>
       </c>
-      <c r="L4" s="80"/>
+      <c r="L4" s="81"/>
       <c r="M4" s="64">
         <f t="shared" si="3"/>
         <v>0.83333333333333337</v>
@@ -11678,10 +11681,10 @@
       <c r="J5" s="11">
         <v>18</v>
       </c>
-      <c r="K5" s="79">
+      <c r="K5" s="80">
         <v>3</v>
       </c>
-      <c r="L5" s="80"/>
+      <c r="L5" s="81"/>
       <c r="M5" s="64">
         <f t="shared" si="3"/>
         <v>0.8571428571428571</v>
@@ -11754,10 +11757,10 @@
       <c r="J6" s="20">
         <v>44</v>
       </c>
-      <c r="K6" s="85">
+      <c r="K6" s="82">
         <v>11</v>
       </c>
-      <c r="L6" s="86"/>
+      <c r="L6" s="83"/>
       <c r="M6" s="64">
         <f t="shared" si="3"/>
         <v>0.8</v>
@@ -11830,10 +11833,10 @@
       <c r="J7" s="16">
         <v>10</v>
       </c>
-      <c r="K7" s="83">
+      <c r="K7" s="84">
         <v>1</v>
       </c>
-      <c r="L7" s="84"/>
+      <c r="L7" s="85"/>
       <c r="M7" s="64">
         <f t="shared" si="3"/>
         <v>0.90909090909090906</v>
@@ -11906,10 +11909,10 @@
       <c r="J8" s="27">
         <v>8</v>
       </c>
-      <c r="K8" s="87">
+      <c r="K8" s="92">
         <v>1</v>
       </c>
-      <c r="L8" s="88"/>
+      <c r="L8" s="93"/>
       <c r="M8" s="64">
         <f t="shared" si="3"/>
         <v>0.88888888888888884</v>
@@ -12058,10 +12061,10 @@
       <c r="J10" s="16">
         <v>112</v>
       </c>
-      <c r="K10" s="83">
+      <c r="K10" s="84">
         <v>2</v>
       </c>
-      <c r="L10" s="84"/>
+      <c r="L10" s="85"/>
       <c r="M10" s="64">
         <f t="shared" si="3"/>
         <v>0.98245614035087714</v>
@@ -12134,10 +12137,10 @@
       <c r="J11" s="11">
         <v>77</v>
       </c>
-      <c r="K11" s="79">
+      <c r="K11" s="80">
         <v>1</v>
       </c>
-      <c r="L11" s="80"/>
+      <c r="L11" s="81"/>
       <c r="M11" s="64">
         <f t="shared" si="3"/>
         <v>0.98717948717948723</v>
@@ -12210,10 +12213,10 @@
       <c r="J12" s="11">
         <v>61</v>
       </c>
-      <c r="K12" s="79">
+      <c r="K12" s="80">
         <v>4</v>
       </c>
-      <c r="L12" s="80"/>
+      <c r="L12" s="81"/>
       <c r="M12" s="64">
         <f t="shared" si="3"/>
         <v>0.93846153846153846</v>
@@ -12286,10 +12289,10 @@
       <c r="J13" s="20">
         <v>64</v>
       </c>
-      <c r="K13" s="85">
+      <c r="K13" s="82">
         <v>1</v>
       </c>
-      <c r="L13" s="86"/>
+      <c r="L13" s="83"/>
       <c r="M13" s="64">
         <f t="shared" si="3"/>
         <v>0.98461538461538467</v>
@@ -12362,10 +12365,10 @@
       <c r="J14" s="16">
         <v>21</v>
       </c>
-      <c r="K14" s="83">
+      <c r="K14" s="84">
         <v>1</v>
       </c>
-      <c r="L14" s="84"/>
+      <c r="L14" s="85"/>
       <c r="M14" s="64">
         <f t="shared" si="3"/>
         <v>0.95454545454545459</v>
@@ -12437,10 +12440,10 @@
       <c r="J15" s="34">
         <v>28</v>
       </c>
-      <c r="K15" s="89">
+      <c r="K15" s="86">
         <v>0</v>
       </c>
-      <c r="L15" s="90"/>
+      <c r="L15" s="87"/>
       <c r="M15" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -12513,10 +12516,10 @@
       <c r="J16" s="40">
         <v>23</v>
       </c>
-      <c r="K16" s="91">
+      <c r="K16" s="88">
         <v>1</v>
       </c>
-      <c r="L16" s="92"/>
+      <c r="L16" s="89"/>
       <c r="M16" s="64">
         <f t="shared" si="3"/>
         <v>0.95833333333333337</v>
@@ -12665,10 +12668,10 @@
       <c r="J18" s="16">
         <v>133</v>
       </c>
-      <c r="K18" s="83">
+      <c r="K18" s="84">
         <v>2</v>
       </c>
-      <c r="L18" s="84"/>
+      <c r="L18" s="85"/>
       <c r="M18" s="64">
         <f t="shared" si="3"/>
         <v>0.98518518518518516</v>
@@ -12741,10 +12744,10 @@
       <c r="J19" s="11">
         <v>111</v>
       </c>
-      <c r="K19" s="79">
+      <c r="K19" s="80">
         <v>1</v>
       </c>
-      <c r="L19" s="80"/>
+      <c r="L19" s="81"/>
       <c r="M19" s="64">
         <f t="shared" si="3"/>
         <v>0.9910714285714286</v>
@@ -12817,10 +12820,10 @@
       <c r="J20" s="11">
         <v>76</v>
       </c>
-      <c r="K20" s="79">
+      <c r="K20" s="80">
         <v>1</v>
       </c>
-      <c r="L20" s="80"/>
+      <c r="L20" s="81"/>
       <c r="M20" s="64">
         <f t="shared" si="3"/>
         <v>0.98701298701298701</v>
@@ -12892,10 +12895,10 @@
       <c r="J21" s="11">
         <v>43</v>
       </c>
-      <c r="K21" s="79">
+      <c r="K21" s="80">
         <v>2</v>
       </c>
-      <c r="L21" s="80"/>
+      <c r="L21" s="81"/>
       <c r="M21" s="64">
         <f t="shared" si="3"/>
         <v>0.9555555555555556</v>
@@ -12968,10 +12971,10 @@
       <c r="J22" s="20">
         <v>86</v>
       </c>
-      <c r="K22" s="85">
+      <c r="K22" s="82">
         <v>1</v>
       </c>
-      <c r="L22" s="86"/>
+      <c r="L22" s="83"/>
       <c r="M22" s="64">
         <f t="shared" si="3"/>
         <v>0.9885057471264368</v>
@@ -13044,10 +13047,10 @@
       <c r="J23" s="16">
         <v>26</v>
       </c>
-      <c r="K23" s="83">
+      <c r="K23" s="84">
         <v>1</v>
       </c>
-      <c r="L23" s="84"/>
+      <c r="L23" s="85"/>
       <c r="M23" s="64">
         <f t="shared" si="3"/>
         <v>0.96296296296296291</v>
@@ -13119,10 +13122,10 @@
       <c r="J24" s="34">
         <v>30</v>
       </c>
-      <c r="K24" s="89">
+      <c r="K24" s="86">
         <v>0</v>
       </c>
-      <c r="L24" s="90"/>
+      <c r="L24" s="87"/>
       <c r="M24" s="64">
         <f t="shared" si="3"/>
         <v>1</v>
@@ -13195,10 +13198,10 @@
       <c r="J25" s="49">
         <v>43</v>
       </c>
-      <c r="K25" s="93">
+      <c r="K25" s="76">
         <v>2</v>
       </c>
-      <c r="L25" s="94"/>
+      <c r="L25" s="77"/>
       <c r="M25" s="64">
         <f t="shared" si="3"/>
         <v>0.9555555555555556</v>
@@ -13270,11 +13273,11 @@
       <c r="J26" s="56">
         <v>143</v>
       </c>
-      <c r="K26" s="95">
+      <c r="K26" s="78">
         <f>I26-J26</f>
         <v>6</v>
       </c>
-      <c r="L26" s="96"/>
+      <c r="L26" s="79"/>
       <c r="M26" s="64">
         <f t="shared" si="3"/>
         <v>0.95973154362416102</v>
@@ -13921,7 +13924,7 @@
       </c>
     </row>
     <row r="35" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
+      <c r="A35" s="43" t="s">
         <v>47</v>
       </c>
       <c r="B35" t="s">
@@ -13952,10 +13955,10 @@
       <c r="J35">
         <v>134</v>
       </c>
-      <c r="K35" s="76">
+      <c r="K35" s="94">
         <v>27</v>
       </c>
-      <c r="L35" s="76"/>
+      <c r="L35" s="94"/>
       <c r="M35" s="64">
         <f t="shared" si="3"/>
         <v>0.83229813664596275</v>
@@ -13994,7 +13997,7 @@
       </c>
     </row>
     <row r="36" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
+      <c r="A36" s="43" t="s">
         <v>47</v>
       </c>
       <c r="B36" t="s">
@@ -14025,10 +14028,10 @@
       <c r="J36">
         <v>118</v>
       </c>
-      <c r="K36" s="77">
+      <c r="K36" s="95">
         <v>33</v>
       </c>
-      <c r="L36" s="77"/>
+      <c r="L36" s="95"/>
       <c r="M36" s="64">
         <f t="shared" si="3"/>
         <v>0.7814569536423841</v>
@@ -14067,7 +14070,7 @@
       </c>
     </row>
     <row r="37" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
+      <c r="A37" s="43" t="s">
         <v>47</v>
       </c>
       <c r="B37" t="s">
@@ -14098,10 +14101,10 @@
       <c r="J37">
         <v>86</v>
       </c>
-      <c r="K37" s="77">
+      <c r="K37" s="95">
         <v>40</v>
       </c>
-      <c r="L37" s="77"/>
+      <c r="L37" s="95"/>
       <c r="M37" s="64">
         <f t="shared" si="3"/>
         <v>0.68253968253968256</v>
@@ -14140,7 +14143,7 @@
       </c>
     </row>
     <row r="38" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
+      <c r="A38" s="43" t="s">
         <v>47</v>
       </c>
       <c r="B38" t="s">
@@ -14171,10 +14174,10 @@
       <c r="J38">
         <v>91</v>
       </c>
-      <c r="K38" s="77">
+      <c r="K38" s="95">
         <v>35</v>
       </c>
-      <c r="L38" s="77"/>
+      <c r="L38" s="95"/>
       <c r="M38" s="64">
         <f t="shared" si="3"/>
         <v>0.72222222222222221</v>
@@ -14213,7 +14216,7 @@
       </c>
     </row>
     <row r="39" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
+      <c r="A39" s="43" t="s">
         <v>47</v>
       </c>
       <c r="B39" t="s">
@@ -14244,10 +14247,10 @@
       <c r="J39">
         <v>92</v>
       </c>
-      <c r="K39" s="77">
+      <c r="K39" s="95">
         <v>38</v>
       </c>
-      <c r="L39" s="77"/>
+      <c r="L39" s="95"/>
       <c r="M39" s="64">
         <f t="shared" si="3"/>
         <v>0.70769230769230773</v>
@@ -14286,7 +14289,7 @@
       </c>
     </row>
     <row r="40" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
+      <c r="A40" s="43" t="s">
         <v>47</v>
       </c>
       <c r="B40" t="s">
@@ -14317,10 +14320,10 @@
       <c r="J40">
         <v>53</v>
       </c>
-      <c r="K40" s="77">
+      <c r="K40" s="95">
         <v>23</v>
       </c>
-      <c r="L40" s="77"/>
+      <c r="L40" s="95"/>
       <c r="M40" s="64">
         <f t="shared" si="3"/>
         <v>0.69736842105263153</v>
@@ -14359,7 +14362,7 @@
       </c>
     </row>
     <row r="41" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
+      <c r="A41" s="43" t="s">
         <v>47</v>
       </c>
       <c r="B41" t="s">
@@ -14390,10 +14393,10 @@
       <c r="J41">
         <v>29</v>
       </c>
-      <c r="K41" s="77">
+      <c r="K41" s="95">
         <v>5</v>
       </c>
-      <c r="L41" s="77"/>
+      <c r="L41" s="95"/>
       <c r="M41" s="64">
         <f t="shared" si="3"/>
         <v>0.8529411764705882</v>
@@ -14432,7 +14435,7 @@
       </c>
     </row>
     <row r="42" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
+      <c r="A42" s="43" t="s">
         <v>47</v>
       </c>
       <c r="B42" t="s">
@@ -14463,10 +14466,10 @@
       <c r="J42">
         <v>22</v>
       </c>
-      <c r="K42" s="77">
+      <c r="K42" s="95">
         <v>7</v>
       </c>
-      <c r="L42" s="77"/>
+      <c r="L42" s="95"/>
       <c r="M42" s="64">
         <f t="shared" si="3"/>
         <v>0.75862068965517238</v>
@@ -14505,7 +14508,7 @@
       </c>
     </row>
     <row r="43" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
+      <c r="A43" s="43" t="s">
         <v>47</v>
       </c>
       <c r="B43" t="s">
@@ -14536,10 +14539,10 @@
       <c r="J43">
         <v>40</v>
       </c>
-      <c r="K43" s="78">
+      <c r="K43" s="96">
         <v>20</v>
       </c>
-      <c r="L43" s="78"/>
+      <c r="L43" s="96"/>
       <c r="M43" s="64">
         <f t="shared" si="3"/>
         <v>0.66666666666666663</v>
@@ -15261,28 +15264,717 @@
         <v>0.97674418604651159</v>
       </c>
     </row>
+    <row r="53" spans="1:22" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B53" t="s">
+        <v>22</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D53" s="9">
+        <v>13</v>
+      </c>
+      <c r="E53" s="10">
+        <v>13</v>
+      </c>
+      <c r="F53" s="11">
+        <f>D53-E53</f>
+        <v>0</v>
+      </c>
+      <c r="G53" s="64">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H53" s="9">
+        <f>E53*4*3</f>
+        <v>156</v>
+      </c>
+      <c r="I53" s="11">
+        <f>J53+K53</f>
+        <v>101</v>
+      </c>
+      <c r="J53" s="70">
+        <v>85</v>
+      </c>
+      <c r="K53" s="74">
+        <v>16</v>
+      </c>
+      <c r="L53" s="75"/>
+      <c r="M53" s="64">
+        <f t="shared" si="3"/>
+        <v>0.84158415841584155</v>
+      </c>
+      <c r="N53" s="12">
+        <v>65</v>
+      </c>
+      <c r="O53" s="66">
+        <f t="shared" si="4"/>
+        <v>0.76470588235294112</v>
+      </c>
+      <c r="P53" s="11">
+        <v>57</v>
+      </c>
+      <c r="Q53" s="66">
+        <f t="shared" si="5"/>
+        <v>0.6705882352941176</v>
+      </c>
+      <c r="R53" s="11">
+        <v>11</v>
+      </c>
+      <c r="S53" s="67">
+        <f t="shared" si="6"/>
+        <v>0.12941176470588237</v>
+      </c>
+      <c r="T53" s="9">
+        <v>21</v>
+      </c>
+      <c r="U53" s="66">
+        <f t="shared" si="7"/>
+        <v>0.24705882352941178</v>
+      </c>
+      <c r="V53" s="68">
+        <f t="shared" si="8"/>
+        <v>0.75294117647058822</v>
+      </c>
+    </row>
+    <row r="54" spans="1:22" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B54" t="s">
+        <v>22</v>
+      </c>
+      <c r="C54" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D54" s="14">
+        <v>13</v>
+      </c>
+      <c r="E54" s="15">
+        <v>13</v>
+      </c>
+      <c r="F54" s="11">
+        <f t="shared" ref="F54:F57" si="26">D54-E54</f>
+        <v>0</v>
+      </c>
+      <c r="G54" s="64">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H54" s="14">
+        <f>E54*4*2</f>
+        <v>104</v>
+      </c>
+      <c r="I54" s="11">
+        <f>J54+K54</f>
+        <v>105</v>
+      </c>
+      <c r="J54" s="70">
+        <v>82</v>
+      </c>
+      <c r="K54" s="74">
+        <v>23</v>
+      </c>
+      <c r="L54" s="75"/>
+      <c r="M54" s="64">
+        <f t="shared" si="3"/>
+        <v>0.78095238095238095</v>
+      </c>
+      <c r="N54" s="17">
+        <v>106</v>
+      </c>
+      <c r="O54" s="66">
+        <f t="shared" si="4"/>
+        <v>1.2926829268292683</v>
+      </c>
+      <c r="P54" s="16">
+        <v>190</v>
+      </c>
+      <c r="Q54" s="66">
+        <f t="shared" si="5"/>
+        <v>2.3170731707317072</v>
+      </c>
+      <c r="R54" s="16">
+        <v>8</v>
+      </c>
+      <c r="S54" s="67">
+        <f t="shared" si="6"/>
+        <v>9.7560975609756101E-2</v>
+      </c>
+      <c r="T54" s="14">
+        <v>12</v>
+      </c>
+      <c r="U54" s="66">
+        <f t="shared" si="7"/>
+        <v>0.14634146341463414</v>
+      </c>
+      <c r="V54" s="68">
+        <f t="shared" si="8"/>
+        <v>0.85365853658536583</v>
+      </c>
+    </row>
+    <row r="55" spans="1:22" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B55" t="s">
+        <v>22</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D55" s="9">
+        <v>13</v>
+      </c>
+      <c r="E55" s="10">
+        <v>13</v>
+      </c>
+      <c r="F55" s="11">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="G55" s="64">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H55" s="9">
+        <f>E55*4*2</f>
+        <v>104</v>
+      </c>
+      <c r="I55" s="11">
+        <f>J55+K55</f>
+        <v>72</v>
+      </c>
+      <c r="J55" s="70">
+        <v>56</v>
+      </c>
+      <c r="K55" s="74">
+        <v>16</v>
+      </c>
+      <c r="L55" s="75"/>
+      <c r="M55" s="64">
+        <f t="shared" si="3"/>
+        <v>0.77777777777777779</v>
+      </c>
+      <c r="N55" s="12">
+        <v>119</v>
+      </c>
+      <c r="O55" s="66">
+        <f t="shared" si="4"/>
+        <v>2.125</v>
+      </c>
+      <c r="P55" s="11">
+        <v>61</v>
+      </c>
+      <c r="Q55" s="66">
+        <f t="shared" si="5"/>
+        <v>1.0892857142857142</v>
+      </c>
+      <c r="R55" s="11">
+        <v>5</v>
+      </c>
+      <c r="S55" s="67">
+        <f t="shared" si="6"/>
+        <v>8.9285714285714288E-2</v>
+      </c>
+      <c r="T55" s="9">
+        <v>8</v>
+      </c>
+      <c r="U55" s="66">
+        <f t="shared" si="7"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="V55" s="68">
+        <f t="shared" si="8"/>
+        <v>0.85714285714285721</v>
+      </c>
+    </row>
+    <row r="56" spans="1:22" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B56" t="s">
+        <v>22</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D56" s="9">
+        <v>13</v>
+      </c>
+      <c r="E56" s="10">
+        <v>12</v>
+      </c>
+      <c r="F56" s="11">
+        <f t="shared" si="26"/>
+        <v>1</v>
+      </c>
+      <c r="G56" s="64">
+        <f t="shared" si="1"/>
+        <v>0.92307692307692313</v>
+      </c>
+      <c r="H56" s="9">
+        <f>E56*4*2</f>
+        <v>96</v>
+      </c>
+      <c r="I56" s="11">
+        <f t="shared" ref="I56:I61" si="27">J56+K56</f>
+        <v>63</v>
+      </c>
+      <c r="J56" s="70">
+        <v>53</v>
+      </c>
+      <c r="K56" s="74">
+        <v>10</v>
+      </c>
+      <c r="L56" s="75"/>
+      <c r="M56" s="64">
+        <f t="shared" si="3"/>
+        <v>0.84126984126984128</v>
+      </c>
+      <c r="N56" s="12">
+        <v>120</v>
+      </c>
+      <c r="O56" s="66">
+        <f t="shared" si="4"/>
+        <v>2.2641509433962264</v>
+      </c>
+      <c r="P56" s="11">
+        <v>50</v>
+      </c>
+      <c r="Q56" s="66">
+        <f t="shared" si="5"/>
+        <v>0.94339622641509435</v>
+      </c>
+      <c r="R56" s="11">
+        <v>0</v>
+      </c>
+      <c r="S56" s="67">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="T56" s="9">
+        <v>8</v>
+      </c>
+      <c r="U56" s="66">
+        <f t="shared" si="7"/>
+        <v>0.15094339622641509</v>
+      </c>
+      <c r="V56" s="68">
+        <f t="shared" si="8"/>
+        <v>0.84905660377358494</v>
+      </c>
+    </row>
+    <row r="57" spans="1:22" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B57" t="s">
+        <v>35</v>
+      </c>
+      <c r="C57" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D57" s="9">
+        <v>10</v>
+      </c>
+      <c r="E57" s="10">
+        <v>10</v>
+      </c>
+      <c r="F57" s="11">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="G57" s="64">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H57" s="9">
+        <f>E57*3*2</f>
+        <v>60</v>
+      </c>
+      <c r="I57" s="11">
+        <f t="shared" si="27"/>
+        <v>86</v>
+      </c>
+      <c r="J57" s="70">
+        <v>73</v>
+      </c>
+      <c r="K57" s="74">
+        <v>13</v>
+      </c>
+      <c r="L57" s="75"/>
+      <c r="M57" s="64">
+        <f t="shared" si="3"/>
+        <v>0.84883720930232553</v>
+      </c>
+      <c r="N57" s="12">
+        <v>103</v>
+      </c>
+      <c r="O57" s="66">
+        <f t="shared" si="4"/>
+        <v>1.4109589041095891</v>
+      </c>
+      <c r="P57" s="11">
+        <v>102</v>
+      </c>
+      <c r="Q57" s="66">
+        <f t="shared" si="5"/>
+        <v>1.3972602739726028</v>
+      </c>
+      <c r="R57" s="11">
+        <v>29</v>
+      </c>
+      <c r="S57" s="67">
+        <f t="shared" si="6"/>
+        <v>0.39726027397260272</v>
+      </c>
+      <c r="T57" s="9">
+        <v>12</v>
+      </c>
+      <c r="U57" s="66">
+        <f t="shared" si="7"/>
+        <v>0.16438356164383561</v>
+      </c>
+      <c r="V57" s="68">
+        <f t="shared" si="8"/>
+        <v>0.83561643835616439</v>
+      </c>
+    </row>
+    <row r="58" spans="1:22" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B58" t="s">
+        <v>27</v>
+      </c>
+      <c r="C58" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D58" s="18">
+        <v>13</v>
+      </c>
+      <c r="E58" s="19">
+        <v>13</v>
+      </c>
+      <c r="F58" s="20">
+        <f>D58-E58</f>
+        <v>0</v>
+      </c>
+      <c r="G58" s="64">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H58" s="18">
+        <f>E58*8*2</f>
+        <v>208</v>
+      </c>
+      <c r="I58" s="11">
+        <f t="shared" si="27"/>
+        <v>65</v>
+      </c>
+      <c r="J58" s="71">
+        <v>55</v>
+      </c>
+      <c r="K58" s="74">
+        <v>10</v>
+      </c>
+      <c r="L58" s="75"/>
+      <c r="M58" s="64">
+        <f t="shared" si="3"/>
+        <v>0.84615384615384615</v>
+      </c>
+      <c r="N58" s="21">
+        <v>3</v>
+      </c>
+      <c r="O58" s="66">
+        <f t="shared" si="4"/>
+        <v>5.4545454545454543E-2</v>
+      </c>
+      <c r="P58" s="20">
+        <v>0</v>
+      </c>
+      <c r="Q58" s="66">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R58" s="20">
+        <v>6</v>
+      </c>
+      <c r="S58" s="67">
+        <f t="shared" si="6"/>
+        <v>0.10909090909090909</v>
+      </c>
+      <c r="T58" s="18">
+        <v>6</v>
+      </c>
+      <c r="U58" s="66">
+        <f t="shared" si="7"/>
+        <v>0.10909090909090909</v>
+      </c>
+      <c r="V58" s="68">
+        <f t="shared" si="8"/>
+        <v>0.89090909090909087</v>
+      </c>
+    </row>
+    <row r="59" spans="1:22" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B59" t="s">
+        <v>27</v>
+      </c>
+      <c r="C59" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="D59" s="14">
+        <v>13</v>
+      </c>
+      <c r="E59" s="15">
+        <v>13</v>
+      </c>
+      <c r="F59" s="20">
+        <f t="shared" ref="F59:F60" si="28">D59-E59</f>
+        <v>0</v>
+      </c>
+      <c r="G59" s="64">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="H59" s="14">
+        <f>E59*4*2</f>
+        <v>104</v>
+      </c>
+      <c r="I59" s="11">
+        <f t="shared" si="27"/>
+        <v>45</v>
+      </c>
+      <c r="J59" s="70">
+        <v>36</v>
+      </c>
+      <c r="K59" s="74">
+        <v>9</v>
+      </c>
+      <c r="L59" s="75"/>
+      <c r="M59" s="64">
+        <f t="shared" si="3"/>
+        <v>0.8</v>
+      </c>
+      <c r="N59" s="17">
+        <v>0</v>
+      </c>
+      <c r="O59" s="66">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="P59" s="16">
+        <v>0</v>
+      </c>
+      <c r="Q59" s="66">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R59" s="16">
+        <v>7</v>
+      </c>
+      <c r="S59" s="67">
+        <f t="shared" si="6"/>
+        <v>0.19444444444444445</v>
+      </c>
+      <c r="T59" s="14">
+        <v>1</v>
+      </c>
+      <c r="U59" s="66">
+        <f t="shared" si="7"/>
+        <v>2.7777777777777776E-2</v>
+      </c>
+      <c r="V59" s="68">
+        <f t="shared" si="8"/>
+        <v>0.97222222222222221</v>
+      </c>
+    </row>
+    <row r="60" spans="1:22" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B60" t="s">
+        <v>27</v>
+      </c>
+      <c r="C60" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="D60" s="32">
+        <v>13</v>
+      </c>
+      <c r="E60" s="33">
+        <v>8</v>
+      </c>
+      <c r="F60" s="20">
+        <f t="shared" si="28"/>
+        <v>5</v>
+      </c>
+      <c r="G60" s="64">
+        <f t="shared" si="1"/>
+        <v>0.61538461538461542</v>
+      </c>
+      <c r="H60" s="32">
+        <f>E60*4*2</f>
+        <v>64</v>
+      </c>
+      <c r="I60" s="11">
+        <f t="shared" si="27"/>
+        <v>19</v>
+      </c>
+      <c r="J60" s="72">
+        <v>12</v>
+      </c>
+      <c r="K60" s="74">
+        <v>7</v>
+      </c>
+      <c r="L60" s="75"/>
+      <c r="M60" s="64">
+        <f t="shared" si="3"/>
+        <v>0.63157894736842102</v>
+      </c>
+      <c r="N60" s="35">
+        <v>0</v>
+      </c>
+      <c r="O60" s="66">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="P60" s="34">
+        <v>0</v>
+      </c>
+      <c r="Q60" s="66">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R60" s="34">
+        <v>1</v>
+      </c>
+      <c r="S60" s="67">
+        <f t="shared" si="6"/>
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="T60" s="32">
+        <v>0</v>
+      </c>
+      <c r="U60" s="66">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="V60" s="68">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:22" ht="46.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B61" t="s">
+        <v>30</v>
+      </c>
+      <c r="C61" s="44" t="s">
+        <v>31</v>
+      </c>
+      <c r="D61" s="45">
+        <v>8</v>
+      </c>
+      <c r="E61" s="46">
+        <v>7</v>
+      </c>
+      <c r="F61" s="47">
+        <f>D61-E61</f>
+        <v>1</v>
+      </c>
+      <c r="G61" s="64">
+        <f t="shared" si="1"/>
+        <v>0.875</v>
+      </c>
+      <c r="H61" s="45">
+        <f>E61*4*2</f>
+        <v>56</v>
+      </c>
+      <c r="I61" s="11">
+        <f t="shared" si="27"/>
+        <v>33</v>
+      </c>
+      <c r="J61" s="73">
+        <v>20</v>
+      </c>
+      <c r="K61" s="74">
+        <v>13</v>
+      </c>
+      <c r="L61" s="75"/>
+      <c r="M61" s="64">
+        <f t="shared" si="3"/>
+        <v>0.60606060606060608</v>
+      </c>
+      <c r="N61" s="35">
+        <v>0</v>
+      </c>
+      <c r="O61" s="66">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="P61" s="34">
+        <v>0</v>
+      </c>
+      <c r="Q61" s="66">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R61" s="49">
+        <v>0</v>
+      </c>
+      <c r="S61" s="67">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="T61" s="51">
+        <v>1</v>
+      </c>
+      <c r="U61" s="66">
+        <f t="shared" si="7"/>
+        <v>0.05</v>
+      </c>
+      <c r="V61" s="68">
+        <f t="shared" si="8"/>
+        <v>0.95</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="52">
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="K18:L18"/>
+  <mergeCells count="61">
+    <mergeCell ref="K58:L58"/>
+    <mergeCell ref="K59:L59"/>
+    <mergeCell ref="K60:L60"/>
+    <mergeCell ref="K61:L61"/>
+    <mergeCell ref="K53:L53"/>
+    <mergeCell ref="K54:L54"/>
+    <mergeCell ref="K55:L55"/>
+    <mergeCell ref="K56:L56"/>
+    <mergeCell ref="K57:L57"/>
+    <mergeCell ref="K49:L49"/>
+    <mergeCell ref="K50:L50"/>
+    <mergeCell ref="K51:L51"/>
+    <mergeCell ref="K52:L52"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="K36:L36"/>
+    <mergeCell ref="K37:L37"/>
+    <mergeCell ref="K38:L38"/>
+    <mergeCell ref="K39:L39"/>
+    <mergeCell ref="K40:L40"/>
+    <mergeCell ref="K41:L41"/>
+    <mergeCell ref="K42:L42"/>
+    <mergeCell ref="K43:L43"/>
+    <mergeCell ref="K44:L44"/>
+    <mergeCell ref="K45:L45"/>
+    <mergeCell ref="K46:L46"/>
     <mergeCell ref="K47:L47"/>
     <mergeCell ref="K48:L48"/>
     <mergeCell ref="K12:L12"/>
@@ -15299,22 +15991,26 @@
     <mergeCell ref="K11:L11"/>
     <mergeCell ref="K24:L24"/>
     <mergeCell ref="K13:L13"/>
-    <mergeCell ref="K49:L49"/>
-    <mergeCell ref="K50:L50"/>
-    <mergeCell ref="K51:L51"/>
-    <mergeCell ref="K52:L52"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="K36:L36"/>
-    <mergeCell ref="K37:L37"/>
-    <mergeCell ref="K38:L38"/>
-    <mergeCell ref="K39:L39"/>
-    <mergeCell ref="K40:L40"/>
-    <mergeCell ref="K41:L41"/>
-    <mergeCell ref="K42:L42"/>
-    <mergeCell ref="K43:L43"/>
-    <mergeCell ref="K44:L44"/>
-    <mergeCell ref="K45:L45"/>
-    <mergeCell ref="K46:L46"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="K30:L30"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>